<commit_message>
Synchronize final REB consensus results
Update the README and final Supplementary Data 1 and 4 to the adjudicated 76-study consensus.
</commit_message>
<xml_diff>
--- a/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
+++ b/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0a33ee533866490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="Re63a403c9f4a421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="R95e921d086c34558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R172d3529921d4145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="R19a9ff3cfd084280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Raadded7f7dcf4f05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="R785244b215104258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R6094e63dac664d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="Rc0634c91c2054d7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="R47325c4e312a4f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="R6b28b52cc3c544b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="R0b6c0a96bd164107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R7fa5aaa9b2fc48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rdd188596fd414cc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="R7a33f904089c4191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Re118a346c4b94535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R974d5b2923484ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R44112fb8a30d4985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R09dacb57584b4f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R154999075af64e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R8e3be05f19484ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb705d1291f0b49ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R94f707ed863b4e4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="Rec1cc6967a2944ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Rf21b7ac4ca5e49d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="R758dee57a6ec4ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R81109aaaeaa24588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="Ra07359923a6f4c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Rdf72f128c62f42d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="Rd244073ab7794344"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Rbe37bb6646f14035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R6de5bbe6404f43b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rba3fbdf31a744d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="Rbbd0730fa0ad4579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Recbfc27fa4244023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="Rd0cfec9df75a44f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="Re001d9855fe3499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R5efd07df9a9c41a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,13 +350,16 @@
         <x:v>76 eligible FDM/FFF wearable-sensor studies</x:v>
       </x:c>
     </x:row>
-    <x:row r="2"/>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+    </x:row>
     <x:row r="3" ht="34" hidden="0" customHeight="1">
       <x:c r="A3" s="5" t="str">
         <x:v>Purpose</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>Structured extraction and source locators for 76 studies. Study REB Profile and Synthesis Summary contain the final adjudicated REB results from Supplementary Data 4.</x:v>
+        <x:v>Structured extraction and source locators for 76 studies. REB Coding, Study REB Profile and Synthesis Summary use the final consensus decisions from Supplementary Data 4.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -380,7 +383,7 @@
         <x:v>Identifiers</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>Synthesis ID 1–76 is consecutive for manuscript use. Stable Study ID preserves traceability to screening files and source PDFs.</x:v>
+        <x:v>Synthesis ID 1-76 is consecutive for manuscript use. Stable Study ID preserves traceability to screening files and source PDFs.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -412,7 +415,7 @@
         <x:v>Assessment terminology</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>Methodological concerns (D1–D7) and wearable applicability (D8) are assessed separately from REB. Historical source-tab identifiers are retained for traceability.</x:v>
+        <x:v>Methodological concerns (D1-D7) and wearable applicability (D8) are assessed separately from REB. Historical source-tab identifiers are retained for traceability.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" hidden="0" customHeight="1">
@@ -444,16 +447,12 @@
         <x:v>Consensus provenance</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>REB Coding retains extraction-stage evidence. Final profiles include 36 L7 recodes (1 to 0). Supplementary Data 4 preserves original reviewer ratings and adjudication.</x:v>
+        <x:v>The final profiles use the finalized L7 decisions in Supplementary Data 4. Article-specific reasons and locators are retained in REB Coding.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="5" t="str">
-        <x:v>Version</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>2026-09-23</x:v>
-      </x:c>
+      <x:c r="A15" s="5"/>
+      <x:c r="B15" s="7"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -481,7 +480,7 @@
         <x:v>REB item</x:v>
       </x:c>
       <x:c r="C1" s="11" t="str">
-        <x:v>Extraction-stage decision</x:v>
+        <x:v>Final REB decision</x:v>
       </x:c>
       <x:c r="D1" s="11" t="str">
         <x:v>Supporting evidence/reason</x:v>
@@ -642,19 +641,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>Embedded assembly is described and used, but no interface-specific integrity or pre/post integration-retention criterion was located.</x:v>
+        <x:v>The authors assess GRF pattern and stance-phase repeatability throughout sequential worn gait cycles and discuss biological variability. This is direct qualitative cross-cycle evaluation, not a retention percentage.</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>PDF pp. 4-15 checked</x:v>
+        <x:v>S001_Main.pdf, physical p. 7 protocol; pp. 13-15, Fig. 7a-b and sequential-gait repeatability discussion.</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Uncertain</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1010,19 +1009,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C24" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>On-body attachment is demonstrated but no quantified interface or pre/post-integration verification.</x:v>
+        <x:v>Section 3.3 reports repeatable resistance changes during repeated hand/finger actions with attached sensors. Qualification does not depend on the separate bench durability or stepping demonstration.</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>PDF pp. 2–13; Figs. 1–8</x:v>
+        <x:v>S004_Main.pdf, physical pp. 11-12, section 3.3/Fig. 7a-e.</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1378,19 +1377,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C40" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>Interface pressure/impedance is quantified and coating cracking after prolonged use is reported.</x:v>
+        <x:v>Physical loading tests use 50-350 g loads; p. 11 says long-term cyclic tests were not performed and that coating can begin to crack after prolonged use.</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>PDF pp. 9-11</x:v>
+        <x:v>S007_Main.pdf, physical pp. 10-11, section 3.2, Figs. 9-10 and Table 3; on-person sections pp. 7-9.</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>Uncertain</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G40" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -1562,19 +1561,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C48" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Whole-insole and with/without surrounding-origami responses quantify integration effects.</x:v>
+        <x:v>Fig. 5 distinguishes plantar pressure conditions. Mechanical loading/calibration is characterized separately.</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>PDF pp. 5–10; Figs. 3–5</x:v>
+        <x:v>S008_Main.pdf, physical pp. 7-9, sensor characterization and Fig. 5.</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G48" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -1930,19 +1929,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C64" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>Sensitivity before and after insole integration is quantitatively compared.</x:v>
+        <x:v>The paper notes some drift/delay when the worn signals return near zero within a gait cycle. The one-hour, 2280-cycle durability comparison belongs to the laboratory sensor test.</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>PDF p. 12, Fig. 9</x:v>
+        <x:v>S011_Main.pdf, physical p. 10, section 3.1.4/Fig. 8; pp. 13-14, section 3.2/Figs. 12-13; p. 6, Fig. 2.</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G64" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
@@ -2114,19 +2113,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C72" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D72" s="12" t="str">
-        <x:v>Electrode/contact impedance and final on-body interface performance are quantified.</x:v>
+        <x:v>Electrodes are swapped sequentially between measurements; exact placement is difficult. Larger electrodes perform better; long-term/multiple-use advantages are prospective.</x:v>
       </x:c>
       <x:c r="E72" s="12" t="str">
-        <x:v>PDF pp. 4–14; Figs. 1–17; Tables 2–3</x:v>
+        <x:v>S012_Main.pdf, physical pp. 12-15, electrode-size results, Fig. 14 and Discussion/Conclusions.</x:v>
       </x:c>
       <x:c r="F72" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G72" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -3402,19 +3401,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C128" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D128" s="12" t="str">
-        <x:v>With/without-foam response time and human-in-loop integrated calibration quantify integration effects.</x:v>
+        <x:v>The authors state sensors were characterized on a test bench. Drift in Fig. 7a is discussed as a greater concern for longer tasks or breaks, while the human trial illustrates in-situ calibration.</x:v>
       </x:c>
       <x:c r="E128" s="12" t="str">
-        <x:v>PDF pp. 5–14; Figs. 5–12</x:v>
+        <x:v>S020_Main.pdf, physical pp. 13-14, human-in-the-loop results and Discussion; Fig. 7a bench characterization.</x:v>
       </x:c>
       <x:c r="F128" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G128" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15" hidden="0" customHeight="1">
@@ -3770,19 +3769,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C144" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D144" s="12" t="str">
-        <x:v>Body-conformable demonstrations do not provide a quantitative attachment/integration endpoint.</x:v>
+        <x:v>Normal walking produces periodic waveforms with uniform amplitude, contrasted with variable limping signals; the sole configuration is shown alongside the worn application.</x:v>
       </x:c>
       <x:c r="E144" s="12" t="str">
-        <x:v>PDF pp. 1–9; Figs. 1–6; cited SI</x:v>
+        <x:v>S022_Main.pdf, physical p. 6, full-body monitoring paragraph; p. 7, Fig. 6h-j. Supplied supplement contains separate bench characterization.</x:v>
       </x:c>
       <x:c r="F144" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G144" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="15" hidden="0" customHeight="1">
@@ -4322,19 +4321,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C168" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D168" s="12" t="str">
-        <x:v>Pre/post insertion calibration and triplicate skin insertions quantify retention/integration.</x:v>
+        <x:v>Three consecutive insertions are performed for each patch. The conclusion explicitly places on-body measurements in future work.</x:v>
       </x:c>
       <x:c r="E168" s="12" t="str">
-        <x:v>PDF pp. 2–10; Figs. 1–6; Table 1; cited SI</x:v>
+        <x:v>S025_Main.pdf, physical pp. 9-11, Fig. 5d, Fig. 6/Table 1 and Conclusions; S025_Supplement_01.pdf, ex-vivo and calibration methods.</x:v>
       </x:c>
       <x:c r="F168" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G168" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
@@ -4690,19 +4689,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C184" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D184" s="12" t="str">
-        <x:v>Raw and glove-mounted sets were compared quantitatively, and a complete glove prototype was demonstrated.</x:v>
+        <x:v>The application section demonstrates a glove prototype and response tracking; it also proposes a per-patient disposable-use model.</x:v>
       </x:c>
       <x:c r="E184" s="12" t="str">
-        <x:v>PDF pp. 4–23; Figs. 3–17; Tables 2–7</x:v>
+        <x:v>S029_Main.pdf, physical pp. 22-23, section 3.6, application feasibility and glove demonstration.</x:v>
       </x:c>
       <x:c r="F184" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G184" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="15" hidden="0" customHeight="1">
@@ -5242,19 +5241,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C208" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D208" s="12" t="str">
-        <x:v>Peel-off force was measured in newtons over time for coated, embedded and unmodified TPE sensing units attached to test tape.</x:v>
+        <x:v>The 1000-cycle experiment reports about 30% initial resistance reduction under specimen pressure loading. Fig. 5 demonstrates body-motion response.</x:v>
       </x:c>
       <x:c r="E208" s="12" t="str">
-        <x:v>Supplementary Fig. S2, SI p. 2</x:v>
+        <x:v>S033_Main.pdf, physical pp. 5-7, Figs. 4e and 5; S033_Supplement_01.pdf, pp. 2-3/Figs. S1-S4; supplied Videos S1-S2.</x:v>
       </x:c>
       <x:c r="F208" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G208" s="12" t="str">
-        <x:v>Supplement verified 2026-09-03</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="15" hidden="0" customHeight="1">
@@ -5426,19 +5425,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C216" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D216" s="12" t="str">
-        <x:v>Repeated washing/carryover of the complete assembled device and modular electrode reuse quantify integration retention.</x:v>
+        <x:v>The authors report no carryover after rinsing. Sweat collection/contact is demonstrated, but the rinse/reuse experiments do not establish a repeatedly attached body-worn assembly.</x:v>
       </x:c>
       <x:c r="E216" s="12" t="str">
-        <x:v>PDF pp. 2–9; Figs. 1–5; cited SI</x:v>
+        <x:v>S034_Main.pdf, physical pp. 8-10, biofluid applications, reuse discussion and Conclusions.</x:v>
       </x:c>
       <x:c r="F216" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G216" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="15" hidden="0" customHeight="1">
@@ -5610,19 +5609,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C224" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D224" s="12" t="str">
-        <x:v>The complete ring underwent quantified bending stability and on-body use.</x:v>
+        <x:v>Ten-day stability follows three daily measurements in artificial sweat, washing and room storage. Fifteen bending cycles are described using the illustrated ring deformation; on-body meal monitoring is separate.</x:v>
       </x:c>
       <x:c r="E224" s="12" t="str">
-        <x:v>PDF pp. 1–5; Figs. 1–4; cited SI</x:v>
+        <x:v>S035_Main.pdf, physical pp. 3-5, stability protocol/Fig. 4a versus on-body Fig. 4b; p. 2, Fig. 1B.</x:v>
       </x:c>
       <x:c r="F224" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G224" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="15" hidden="0" customHeight="1">
@@ -5794,19 +5793,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C232" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D232" s="12" t="str">
-        <x:v>Medical adhesive and on-body use are described, but no prespecified quantitative attachment/integration endpoint or pre/post integration comparison is reported.</x:v>
+        <x:v>The attached sweat-rate device cannot accommodate the entire exercise's perspiration volume; monitoring ends at approximately 2200 seconds because its capacity is insufficient.</x:v>
       </x:c>
       <x:c r="E232" s="12" t="str">
-        <x:v>PDF pp. 2–11; Figs. 1–6; cited SI</x:v>
+        <x:v>S036_Main.pdf, physical p. 3, assembly/cycling protocol; pp. 9-10, on-body section, p. 10 first paragraph/Fig. 6.</x:v>
       </x:c>
       <x:c r="F232" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G232" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="233" ht="15" hidden="0" customHeight="1">
@@ -6162,19 +6161,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C248" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D248" s="12" t="str">
-        <x:v>A glove was demonstrated, but no quantitative pre/post integration comparison or interface endpoint was reported.</x:v>
+        <x:v>The text explicitly reports relatively repeatable resistance responses across all three flexing cycles at the specified positions.</x:v>
       </x:c>
       <x:c r="E248" s="12" t="str">
-        <x:v>PDF pp. 3–12; Figs. 1–11; Table 1</x:v>
+        <x:v>S038_Main.pdf, physical p. 12, section 3.5 and Fig. 11b-c.</x:v>
       </x:c>
       <x:c r="F248" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G248" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="15" hidden="0" customHeight="1">
@@ -6901,16 +6900,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D280" s="12" t="str">
-        <x:v>Human-worn finger-sleeve and insole devices produced quantitative repeated signals; walking outputs were reported at two frequencies.</x:v>
+        <x:v>A Z-shaped spring embedded in the author's insole is assessed during repeated walking at two frequencies; maintained stable voltage is explicitly reported.</x:v>
       </x:c>
       <x:c r="E280" s="12" t="str">
-        <x:v>PDF pp. 2–7; Figs. 3–5; cited Supplementary Figs. S1–S5</x:v>
+        <x:v>S046_Main.pdf, physical pp. 6-7, Fig. 5c-e and application paragraph (printed pp. 1021-1022).</x:v>
       </x:c>
       <x:c r="F280" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G280" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="281" ht="24" hidden="0" customHeight="1">
@@ -7085,16 +7084,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D288" s="12" t="str">
-        <x:v>The complete mask was calibrated at the skin and logged interface pressure during four weeks of wear.</x:v>
+        <x:v>Pressure is recorded to confirm maintenance of 15-25 mmHg; section 3.2.1 reports that mean pressure is maintained through the trial with strap adjustment.</x:v>
       </x:c>
       <x:c r="E288" s="12" t="str">
-        <x:v>PDF pp. 3–13; Figs. 2–12; Table 1</x:v>
+        <x:v>S047_Main.pdf, physical p. 6, clinical protocol; pp. 9-10, section 3.2.1/Fig. 9. The figure shows the initial hour; adjacent text reports trial-period maintenance.</x:v>
       </x:c>
       <x:c r="F288" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G288" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="289" ht="15" hidden="0" customHeight="1">
@@ -7821,16 +7820,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D320" s="12" t="str">
-        <x:v>A hand-worn sensor performed quantitative five-object classification.</x:v>
+        <x:v>The final hand-worn sensor was quantitatively evaluated across five object-manipulation classes.</x:v>
       </x:c>
       <x:c r="E320" s="12" t="str">
-        <x:v>PDF pp. 2–12; Figs. 1–6; cited Supplementary Table S1 and Figs. S1–S21</x:v>
+        <x:v>PDF pp. 10-12; Fig. 6</x:v>
       </x:c>
       <x:c r="F320" s="12" t="str">
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G320" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="321" ht="24" hidden="0" customHeight="1">
@@ -8373,16 +8372,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D344" s="12" t="str">
-        <x:v>The assembled sensor was worn during multiple human motions.</x:v>
+        <x:v>After initial gait adjustment, the body-attached sensor gives a consistent walking output over the reported 10-second interval. Separate 11600-cycle compression is not used for this score.</x:v>
       </x:c>
       <x:c r="E344" s="12" t="str">
-        <x:v>PDF pp. 3–9; Figs. 1–10</x:v>
+        <x:v>S055_Main.pdf, physical p. 7, section 2.6; p. 9, Fig. 6a. Fig. 5g concerns bench durability.</x:v>
       </x:c>
       <x:c r="F344" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G344" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="345" ht="15" hidden="0" customHeight="1">
@@ -8557,16 +8556,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D352" s="12" t="str">
-        <x:v>Complete insole/body/HMI assemblies produced quantitative signals.</x:v>
+        <x:v>The authors evaluate stable signal patterns for repeated calf/neck/larynx actions and stable responses for repeated joint movements in the worn demonstrations.</x:v>
       </x:c>
       <x:c r="E352" s="12" t="str">
-        <x:v>PDF pp. 3–15; Figs. 1–9; Tables 1–2</x:v>
+        <x:v>S056_Main.pdf, physical p. 13, Fig. 11a-h; p. 14, accompanying interpretation and Fig. 12b-c.</x:v>
       </x:c>
       <x:c r="F352" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G352" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="353" ht="15" hidden="0" customHeight="1">
@@ -8741,16 +8740,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D360" s="12" t="str">
-        <x:v>Sensors were quantitatively demonstrated in an insole and on the finger, wrist and throat.</x:v>
+        <x:v>Attached throat sensors produce distinct, reproducible swallowing/coughing profiles; the finger/wrist trials also receive an explicit repeatability assessment.</x:v>
       </x:c>
       <x:c r="E360" s="12" t="str">
-        <x:v>PDF pp. 3–15; Figs. 1–10</x:v>
+        <x:v>S057_Main.pdf, physical pp. 15-16, section 3.3/Fig. 15c-e, especially p. 16 opening paragraph.</x:v>
       </x:c>
       <x:c r="F360" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G360" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="361" ht="15" hidden="0" customHeight="1">
@@ -8925,16 +8924,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D368" s="12" t="str">
-        <x:v>An instrumented insole was tested in six participants using subject-wise validation.</x:v>
+        <x:v>Supplementary Fig. S7c explicitly documents seven days of wear. The paper reports no structural damage, delamination or output failure after the reliability evaluation.</x:v>
       </x:c>
       <x:c r="E368" s="12" t="str">
-        <x:v>PDF pp. 3–13; Figs. 1–8; cited Supplementary Table S1</x:v>
+        <x:v>S058_Supplement_01.docx, Fig. S7c (7-day wear trial); S058_Main.pdf, physical p. 8, reliability discussion, and p. 12, methods.</x:v>
       </x:c>
       <x:c r="F368" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G368" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="369" ht="24" hidden="0" customHeight="1">
@@ -9474,19 +9473,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C392" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D392" s="12" t="str">
-        <x:v>The assembled splint sensor was quantitatively compared in two integration states.</x:v>
+        <x:v>The million-cycle fatigue result is an ANSYS prediction. The worn measurements concern static pressure/antenna response.</x:v>
       </x:c>
       <x:c r="E392" s="12" t="str">
-        <x:v>PDF pp. 2–11; Figs. 1–13; Table 1</x:v>
+        <x:v>S061_Main.pdf, physical p. 6, fatigue simulation; pp. 7-8, Fig. 11/Table 2.</x:v>
       </x:c>
       <x:c r="F392" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G392" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="393" ht="15" hidden="0" customHeight="1">
@@ -10029,16 +10028,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D416" s="12" t="str">
-        <x:v>Complete sensors produced quantitative mouse-click and finger-bending signals.</x:v>
+        <x:v>The authors explicitly evaluate durability during repeated bending and report no delamination or loss of sensitivity, with consistent cycle responses and SNR 34.12 ± 0.72.</x:v>
       </x:c>
       <x:c r="E416" s="12" t="str">
-        <x:v>PDF pp. 2–9; Figs. 1–7</x:v>
+        <x:v>S065_Main.pdf, physical pp. 8-9, section 3.4/Fig. 7c-d.</x:v>
       </x:c>
       <x:c r="F416" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G416" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="417" ht="15" hidden="0" customHeight="1">
@@ -10213,16 +10212,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D424" s="12" t="str">
-        <x:v>The complete wearable system was evaluated in 13 volunteers against BioHarness.</x:v>
+        <x:v>The long-term monitoring section explicitly reports stable amplitude, no drift and no lost periodicity across the recording.</x:v>
       </x:c>
       <x:c r="E424" s="12" t="str">
-        <x:v>PDF pp. 2–8; Figs. 1–8; Table I</x:v>
+        <x:v>S066_Main.pdf, physical p. 5, assembly; pp. 7-8, section V.C, Long-Term Monitoring/Fig. 6.</x:v>
       </x:c>
       <x:c r="F424" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G424" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="425" ht="15" hidden="0" customHeight="1">
@@ -10397,16 +10396,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D432" s="12" t="str">
-        <x:v>A complete insole recorded six activities and supported quantitative classification.</x:v>
+        <x:v>Absolute amplitudes fluctuate, but the text explicitly reports preserved periodicity, inter-peak timing and relative peak relationships across environmental conditions.</x:v>
       </x:c>
       <x:c r="E432" s="12" t="str">
-        <x:v>PDF pp. 2–9; Figs. 1–8</x:v>
+        <x:v>S067_Main.pdf, physical pp. 7-9, Fig. 4e-f and environmental robustness discussion referring to Fig. S6.</x:v>
       </x:c>
       <x:c r="F432" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G432" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="433" ht="15" hidden="0" customHeight="1">
@@ -10581,16 +10580,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D440" s="12" t="str">
-        <x:v>The complete sensor was quantitatively demonstrated on a volunteer and soft robot.</x:v>
+        <x:v>The wrist-mounted sensor is assessed during repeated moderate-force closures; authors describe the waveform as repeatable, with consistent swallowing response in the separate throat configuration.</x:v>
       </x:c>
       <x:c r="E440" s="12" t="str">
-        <x:v>PDF pp. 2–10; Figs. 1–7; Table 1</x:v>
+        <x:v>S068_Main.pdf, physical pp. 8-9, section 3.8/Fig. 7c,e.</x:v>
       </x:c>
       <x:c r="F440" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G440" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="441" ht="15" hidden="0" customHeight="1">
@@ -10762,19 +10761,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C448" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D448" s="12" t="str">
-        <x:v>The printed textile device underwent quantitative adhesion and integrated human-touch tests.</x:v>
+        <x:v>20000 cycles, detergent washing and peel testing assess material/device durability off-body. Supplied video samples show chamber tests, LEDs and table-top finger contact.</x:v>
       </x:c>
       <x:c r="E448" s="12" t="str">
-        <x:v>PDF pp. 2–12; Figs. 1–11; Table 1; cited SI</x:v>
+        <x:v>S069_Main.pdf, physical pp. 11-13, Figs. 10f-g/11; S069_Supplement_01.docx and Supplements 02-04 videos.</x:v>
       </x:c>
       <x:c r="F448" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G448" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="449" ht="15" hidden="0" customHeight="1">
@@ -10949,16 +10948,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D456" s="12" t="str">
-        <x:v>Complete sensors produced quantitative knee and thoracic signals.</x:v>
+        <x:v>The conclusion explicitly reports stable and repeatable response during controlled wearable movement cycles; section V defines the worn protocol.</x:v>
       </x:c>
       <x:c r="E456" s="12" t="str">
-        <x:v>PDF pp. 3–9; Figs. 1–12; Tables I–III</x:v>
+        <x:v>S070_Main.pdf, physical p. 8, section V; p. 9, Fig. 9; p. 10, wearable-validation conclusion.</x:v>
       </x:c>
       <x:c r="F456" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G456" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="457" ht="15" hidden="0" customHeight="1">
@@ -11133,16 +11132,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D464" s="12" t="str">
-        <x:v>The sensor was placed at the plantar interface and tested during gait in five volunteers.</x:v>
+        <x:v>Ten gait cycles per test are analyzed at slow/fast speeds; the authors expressly evaluate stability and reproducibility of the worn sensor across these motion trials.</x:v>
       </x:c>
       <x:c r="E464" s="12" t="str">
-        <x:v>PDF pp. 2–10; Figs. 1–12; Tables 1–2</x:v>
+        <x:v>S071_Main.pdf, physical pp. 9-10, section 3.3/Figs. 11-12.</x:v>
       </x:c>
       <x:c r="F464" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G464" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="465" ht="15" hidden="0" customHeight="1">
@@ -11317,16 +11316,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D472" s="12" t="str">
-        <x:v>Complete sensors were demonstrated on joints and in a glove/robotic-control system.</x:v>
+        <x:v>During worn nominal-angle flexion cycles, peak/interval variability is acknowledged and its effect on the repeated signal trend is evaluated. The response is not claimed to be perfectly repeatable.</x:v>
       </x:c>
       <x:c r="E472" s="12" t="str">
-        <x:v>PDF pp. 2–13; Figs. 1–10; Tables 1–2</x:v>
+        <x:v>S073_Main.pdf, physical pp. 7-8, section 3.2/Fig. 7, especially p. 8 first two paragraphs.</x:v>
       </x:c>
       <x:c r="F472" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G472" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="473" ht="15" hidden="0" customHeight="1">
@@ -11685,16 +11684,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D488" s="12" t="str">
-        <x:v>Tape-integrated sensors produced repeated breathing, knee and elbow signals.</x:v>
+        <x:v>The text explicitly reports the same output for a given angle across all three controlled repetitions, contrasting this with variable returns during unguided movement.</x:v>
       </x:c>
       <x:c r="E488" s="12" t="str">
-        <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
+        <x:v>S075_Main.pdf, physical pp. 7-8, section V; p. 8, Fig. 7c and final controlled-movement paragraph.</x:v>
       </x:c>
       <x:c r="F488" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G488" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="489" ht="24" hidden="0" customHeight="1">
@@ -12053,16 +12052,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D504" s="12" t="str">
-        <x:v>Complete sensors produced quantitative physiological and motion signals.</x:v>
+        <x:v>Section 3.4 explicitly describes consistent response during cyclic pronunciation and subsequent tests, and constant patterns across two extensive chewing cycles.</x:v>
       </x:c>
       <x:c r="E504" s="12" t="str">
-        <x:v>PDF pp. 3–15; Figs. 1–7; Table 1</x:v>
+        <x:v>S077_Main.pdf, physical p. 4, section 2.4 attachment; pp. 11-12, section 3.4/Fig. 6, especially chewing comparison.</x:v>
       </x:c>
       <x:c r="F504" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G504" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="505" ht="15" hidden="0" customHeight="1">
@@ -12237,16 +12236,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D512" s="12" t="str">
-        <x:v>FDM insole and finger-cover devices produced repeated human-motion signals.</x:v>
+        <x:v>Section 2.3 explicitly compares peak values and sizes and describes them as relatively uniform across the finger repetitions.</x:v>
       </x:c>
       <x:c r="E512" s="12" t="str">
-        <x:v>PDF pp. 3–8; Figs. 1–6; Supporting Table S1 cited</x:v>
+        <x:v>S078_Main.pdf, physical p. 7, section 2.3/Fig. 6a-b; S078_Supplement_01.docx.</x:v>
       </x:c>
       <x:c r="F512" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G512" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="513" ht="24" hidden="0" customHeight="1">
@@ -12421,16 +12420,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D520" s="12" t="str">
-        <x:v>Complete sensors and a 4×4 array produced quantitative body/foot-motion signals.</x:v>
+        <x:v>The main text reports about 70% ± 5% resistance change at baseline and minimal change in response to the same bending motions after conditioning.</x:v>
       </x:c>
       <x:c r="E520" s="12" t="str">
-        <x:v>PDF pp. 2–12; Figs. 1–8; Supplementary Figs. S1–S15 cited</x:v>
+        <x:v>S079_Main.pdf, physical p. 10, Fig. 7b; p. 11, section 3.4, paragraph referring to Fig. S15.</x:v>
       </x:c>
       <x:c r="F520" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>Moderate</x:v>
       </x:c>
       <x:c r="G520" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="521" ht="24" hidden="0" customHeight="1">
@@ -12786,19 +12785,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C536" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D536" s="12" t="str">
-        <x:v>Pre/post-embedding spectra and two complete-device clinical procedures provide quantitative integration evidence.</x:v>
+        <x:v>The measured endpoint is timing between sensor response and the clinician's perception in each procedure. Seven compression tests separately characterize sensitivity.</x:v>
       </x:c>
       <x:c r="E536" s="12" t="str">
-        <x:v>PDF pp. 3–7; Figs. 1–8; Table I</x:v>
+        <x:v>S081_Main.pdf, physical pp. 4-5, calibration; pp. 5-7, section IV/Figs. 7-8 and Conclusions.</x:v>
       </x:c>
       <x:c r="F536" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G536" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="537" ht="15" hidden="0" customHeight="1">
@@ -13338,19 +13337,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C560" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D560" s="12" t="str">
-        <x:v>The substrate-integrated sensor underwent repeated loading and generated lumbar-motion signals.</x:v>
+        <x:v>The sensor remains intact against its film substrate after laboratory cycling. Fig. 18 sketches a lumbar use case without a corresponding repeated-wear retention dataset.</x:v>
       </x:c>
       <x:c r="E560" s="12" t="str">
-        <x:v>PDF pp. 2–4, 8–12; Figs. 1–18; Tables 1–2</x:v>
+        <x:v>S085_Main.pdf, physical pp. 3-4, setup/Fig. 4; pp. 9-10, Fig. 15; p. 12, Fig. 18/application discussion.</x:v>
       </x:c>
       <x:c r="F560" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G560" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="561" ht="24" hidden="0" customHeight="1">
@@ -13893,16 +13892,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D584" s="12" t="str">
-        <x:v>Two completed rings were calibrated and used for repeated body-joint measurements.</x:v>
+        <x:v>An additional cyclic test explicitly examines measurement performance; six bends show relatively stable wavelength changes. Repeated calibration tests are also reported.</x:v>
       </x:c>
       <x:c r="E584" s="12" t="str">
-        <x:v>PDF pp. 4–12; Figs. 1–10; Table 1</x:v>
+        <x:v>S088_Main.pdf, physical p. 7, cyclic-elbow paragraph; p. 10, Fig. 8 (the paragraph mislabels its figure reference as Fig. 7).</x:v>
       </x:c>
       <x:c r="F584" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G584" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Final L7 reassessment</x:v>
       </x:c>
     </x:row>
     <x:row r="585" ht="15" hidden="0" customHeight="1">
@@ -29072,7 +29071,7 @@
         <x:v>REB score R</x:v>
       </x:c>
       <x:c r="M1" s="11" t="str">
-        <x:v>L5–L8 count</x:v>
+        <x:v>L5-L8 count</x:v>
       </x:c>
       <x:c r="N1" s="11" t="str">
         <x:v>Unresolved items</x:v>
@@ -29107,21 +29106,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J2" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K2" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L2" s="14" t="n">
-        <x:f>IF(COUNT(D2:K2)=8,SUM(D2:K2)/8,"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M2" s="13" t="n">
-        <x:f>IF(COUNT(H2:K2)=4,SUM(H2:K2),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N2" s="13" t="n">
-        <x:f>COUNTIF(D2:K2,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29160,15 +29156,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L3" s="14" t="n">
-        <x:f>IF(COUNT(D3:K3)=8,SUM(D3:K3)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M3" s="13" t="n">
-        <x:f>IF(COUNT(H3:K3)=4,SUM(H3:K3),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N3" s="13" t="n">
-        <x:f>COUNTIF(D3:K3,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29201,21 +29194,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K4" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="14" t="n">
-        <x:f>IF(COUNT(D4:K4)=8,SUM(D4:K4)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M4" s="13" t="n">
-        <x:f>IF(COUNT(H4:K4)=4,SUM(H4:K4),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N4" s="13" t="n">
-        <x:f>COUNTIF(D4:K4,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29254,15 +29244,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L5" s="14" t="n">
-        <x:f>IF(COUNT(D5:K5)=8,SUM(D5:K5)/8,"Pending")</x:f>
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="M5" s="13" t="n">
-        <x:f>IF(COUNT(H5:K5)=4,SUM(H5:K5),"Pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N5" s="13" t="n">
-        <x:f>COUNTIF(D5:K5,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29295,21 +29282,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J6" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K6" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L6" s="14" t="n">
-        <x:f>IF(COUNT(D6:K6)=8,SUM(D6:K6)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M6" s="13" t="n">
-        <x:f>IF(COUNT(H6:K6)=4,SUM(H6:K6),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N6" s="13" t="n">
-        <x:f>COUNTIF(D6:K6,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29342,21 +29326,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L7" s="14" t="n">
-        <x:f>IF(COUNT(D7:K7)=8,SUM(D7:K7)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M7" s="13" t="n">
-        <x:f>IF(COUNT(H7:K7)=4,SUM(H7:K7),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N7" s="13" t="n">
-        <x:f>COUNTIF(D7:K7,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29395,15 +29376,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L8" s="14" t="n">
-        <x:f>IF(COUNT(D8:K8)=8,SUM(D8:K8)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M8" s="13" t="n">
-        <x:f>IF(COUNT(H8:K8)=4,SUM(H8:K8),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N8" s="13" t="n">
-        <x:f>COUNTIF(D8:K8,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29436,21 +29414,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K9" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L9" s="14" t="n">
-        <x:f>IF(COUNT(D9:K9)=8,SUM(D9:K9)/8,"Pending")</x:f>
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M9" s="13" t="n">
-        <x:f>IF(COUNT(H9:K9)=4,SUM(H9:K9),"Pending")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N9" s="13" t="n">
-        <x:f>COUNTIF(D9:K9,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29483,21 +29458,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L10" s="14" t="n">
-        <x:f>IF(COUNT(D10:K10)=8,SUM(D10:K10)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M10" s="13" t="n">
-        <x:f>IF(COUNT(H10:K10)=4,SUM(H10:K10),"Pending")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N10" s="13" t="n">
-        <x:f>COUNTIF(D10:K10,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29536,15 +29508,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L11" s="14" t="n">
-        <x:f>IF(COUNT(D11:K11)=8,SUM(D11:K11)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M11" s="13" t="n">
-        <x:f>IF(COUNT(H11:K11)=4,SUM(H11:K11),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N11" s="13" t="n">
-        <x:f>COUNTIF(D11:K11,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29583,15 +29552,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="14" t="n">
-        <x:f>IF(COUNT(D12:K12)=8,SUM(D12:K12)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M12" s="13" t="n">
-        <x:f>IF(COUNT(H12:K12)=4,SUM(H12:K12),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N12" s="13" t="n">
-        <x:f>COUNTIF(D12:K12,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29630,15 +29596,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L13" s="14" t="n">
-        <x:f>IF(COUNT(D13:K13)=8,SUM(D13:K13)/8,"Pending")</x:f>
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="M13" s="13" t="n">
-        <x:f>IF(COUNT(H13:K13)=4,SUM(H13:K13),"Pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="13" t="n">
-        <x:f>COUNTIF(D13:K13,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29677,15 +29640,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L14" s="14" t="n">
-        <x:f>IF(COUNT(D14:K14)=8,SUM(D14:K14)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M14" s="13" t="n">
-        <x:f>IF(COUNT(H14:K14)=4,SUM(H14:K14),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N14" s="13" t="n">
-        <x:f>COUNTIF(D14:K14,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29724,15 +29684,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L15" s="14" t="n">
-        <x:f>IF(COUNT(D15:K15)=8,SUM(D15:K15)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M15" s="13" t="n">
-        <x:f>IF(COUNT(H15:K15)=4,SUM(H15:K15),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N15" s="13" t="n">
-        <x:f>COUNTIF(D15:K15,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29771,15 +29728,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L16" s="14" t="n">
-        <x:f>IF(COUNT(D16:K16)=8,SUM(D16:K16)/8,"Pending")</x:f>
         <x:v>0.875</x:v>
       </x:c>
       <x:c r="M16" s="13" t="n">
-        <x:f>IF(COUNT(H16:K16)=4,SUM(H16:K16),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N16" s="13" t="n">
-        <x:f>COUNTIF(D16:K16,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29812,21 +29766,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J17" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K17" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L17" s="14" t="n">
-        <x:f>IF(COUNT(D17:K17)=8,SUM(D17:K17)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M17" s="13" t="n">
-        <x:f>IF(COUNT(H17:K17)=4,SUM(H17:K17),"Pending")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N17" s="13" t="n">
-        <x:f>COUNTIF(D17:K17,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29865,15 +29816,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L18" s="14" t="n">
-        <x:f>IF(COUNT(D18:K18)=8,SUM(D18:K18)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M18" s="13" t="n">
-        <x:f>IF(COUNT(H18:K18)=4,SUM(H18:K18),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N18" s="13" t="n">
-        <x:f>COUNTIF(D18:K18,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29906,21 +29854,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K19" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L19" s="14" t="n">
-        <x:f>IF(COUNT(D19:K19)=8,SUM(D19:K19)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:f>IF(COUNT(H19:K19)=4,SUM(H19:K19),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N19" s="13" t="n">
-        <x:f>COUNTIF(D19:K19,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -29959,15 +29904,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L20" s="14" t="n">
-        <x:f>IF(COUNT(D20:K20)=8,SUM(D20:K20)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M20" s="13" t="n">
-        <x:f>IF(COUNT(H20:K20)=4,SUM(H20:K20),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N20" s="13" t="n">
-        <x:f>COUNTIF(D20:K20,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30006,15 +29948,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L21" s="14" t="n">
-        <x:f>IF(COUNT(D21:K21)=8,SUM(D21:K21)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M21" s="13" t="n">
-        <x:f>IF(COUNT(H21:K21)=4,SUM(H21:K21),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N21" s="13" t="n">
-        <x:f>COUNTIF(D21:K21,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30047,21 +29986,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J22" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K22" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L22" s="14" t="n">
-        <x:f>IF(COUNT(D22:K22)=8,SUM(D22:K22)/8,"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M22" s="13" t="n">
-        <x:f>IF(COUNT(H22:K22)=4,SUM(H22:K22),"Pending")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N22" s="13" t="n">
-        <x:f>COUNTIF(D22:K22,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30100,15 +30036,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L23" s="14" t="n">
-        <x:f>IF(COUNT(D23:K23)=8,SUM(D23:K23)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M23" s="13" t="n">
-        <x:f>IF(COUNT(H23:K23)=4,SUM(H23:K23),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N23" s="13" t="n">
-        <x:f>COUNTIF(D23:K23,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30141,21 +30074,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J24" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K24" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L24" s="14" t="n">
-        <x:f>IF(COUNT(D24:K24)=8,SUM(D24:K24)/8,"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M24" s="13" t="n">
-        <x:f>IF(COUNT(H24:K24)=4,SUM(H24:K24),"Pending")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N24" s="13" t="n">
-        <x:f>COUNTIF(D24:K24,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30194,15 +30124,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L25" s="14" t="n">
-        <x:f>IF(COUNT(D25:K25)=8,SUM(D25:K25)/8,"Pending")</x:f>
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="M25" s="13" t="n">
-        <x:f>IF(COUNT(H25:K25)=4,SUM(H25:K25),"Pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="13" t="n">
-        <x:f>COUNTIF(D25:K25,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30241,15 +30168,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L26" s="14" t="n">
-        <x:f>IF(COUNT(D26:K26)=8,SUM(D26:K26)/8,"Pending")</x:f>
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="M26" s="13" t="n">
-        <x:f>IF(COUNT(H26:K26)=4,SUM(H26:K26),"Pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="13" t="n">
-        <x:f>COUNTIF(D26:K26,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30282,21 +30206,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J27" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K27" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L27" s="14" t="n">
-        <x:f>IF(COUNT(D27:K27)=8,SUM(D27:K27)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:f>IF(COUNT(H27:K27)=4,SUM(H27:K27),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N27" s="13" t="n">
-        <x:f>COUNTIF(D27:K27,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30329,21 +30250,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J28" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K28" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L28" s="14" t="n">
-        <x:f>IF(COUNT(D28:K28)=8,SUM(D28:K28)/8,"Pending")</x:f>
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:f>IF(COUNT(H28:K28)=4,SUM(H28:K28),"Pending")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N28" s="13" t="n">
-        <x:f>COUNTIF(D28:K28,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30376,21 +30294,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J29" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K29" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L29" s="14" t="n">
-        <x:f>IF(COUNT(D29:K29)=8,SUM(D29:K29)/8,"Pending")</x:f>
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M29" s="13" t="n">
-        <x:f>IF(COUNT(H29:K29)=4,SUM(H29:K29),"Pending")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N29" s="13" t="n">
-        <x:f>COUNTIF(D29:K29,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30423,21 +30338,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J30" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K30" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L30" s="14" t="n">
-        <x:f>IF(COUNT(D30:K30)=8,SUM(D30:K30)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M30" s="13" t="n">
-        <x:f>IF(COUNT(H30:K30)=4,SUM(H30:K30),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N30" s="13" t="n">
-        <x:f>COUNTIF(D30:K30,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30476,15 +30388,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L31" s="14" t="n">
-        <x:f>IF(COUNT(D31:K31)=8,SUM(D31:K31)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M31" s="13" t="n">
-        <x:f>IF(COUNT(H31:K31)=4,SUM(H31:K31),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N31" s="13" t="n">
-        <x:f>COUNTIF(D31:K31,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30517,21 +30426,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J32" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K32" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L32" s="14" t="n">
-        <x:f>IF(COUNT(D32:K32)=8,SUM(D32:K32)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M32" s="13" t="n">
-        <x:f>IF(COUNT(H32:K32)=4,SUM(H32:K32),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N32" s="13" t="n">
-        <x:f>COUNTIF(D32:K32,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30570,15 +30476,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L33" s="14" t="n">
-        <x:f>IF(COUNT(D33:K33)=8,SUM(D33:K33)/8,"Pending")</x:f>
         <x:v>0.875</x:v>
       </x:c>
       <x:c r="M33" s="13" t="n">
-        <x:f>IF(COUNT(H33:K33)=4,SUM(H33:K33),"Pending")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="N33" s="13" t="n">
-        <x:f>COUNTIF(D33:K33,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30617,15 +30520,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L34" s="14" t="n">
-        <x:f>IF(COUNT(D34:K34)=8,SUM(D34:K34)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M34" s="13" t="n">
-        <x:f>IF(COUNT(H34:K34)=4,SUM(H34:K34),"Pending")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="13" t="n">
-        <x:f>COUNTIF(D34:K34,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30664,15 +30564,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L35" s="14" t="n">
-        <x:f>IF(COUNT(D35:K35)=8,SUM(D35:K35)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M35" s="13" t="n">
-        <x:f>IF(COUNT(H35:K35)=4,SUM(H35:K35),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N35" s="13" t="n">
-        <x:f>COUNTIF(D35:K35,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30705,21 +30602,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J36" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K36" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L36" s="14" t="n">
-        <x:f>IF(COUNT(D36:K36)=8,SUM(D36:K36)/8,"Pending")</x:f>
-        <x:v>0.375</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M36" s="13" t="n">
-        <x:f>IF(COUNT(H36:K36)=4,SUM(H36:K36),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N36" s="13" t="n">
-        <x:f>COUNTIF(D36:K36,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30752,21 +30646,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J37" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K37" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L37" s="14" t="n">
-        <x:f>IF(COUNT(D37:K37)=8,SUM(D37:K37)/8,"Pending")</x:f>
-        <x:v>0.375</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M37" s="13" t="n">
-        <x:f>IF(COUNT(H37:K37)=4,SUM(H37:K37),"Pending")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N37" s="13" t="n">
-        <x:f>COUNTIF(D37:K37,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30805,15 +30696,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L38" s="14" t="n">
-        <x:f>IF(COUNT(D38:K38)=8,SUM(D38:K38)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M38" s="13" t="n">
-        <x:f>IF(COUNT(H38:K38)=4,SUM(H38:K38),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N38" s="13" t="n">
-        <x:f>COUNTIF(D38:K38,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30852,15 +30740,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L39" s="14" t="n">
-        <x:f>IF(COUNT(D39:K39)=8,SUM(D39:K39)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M39" s="13" t="n">
-        <x:f>IF(COUNT(H39:K39)=4,SUM(H39:K39),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N39" s="13" t="n">
-        <x:f>COUNTIF(D39:K39,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30899,15 +30784,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L40" s="14" t="n">
-        <x:f>IF(COUNT(D40:K40)=8,SUM(D40:K40)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M40" s="13" t="n">
-        <x:f>IF(COUNT(H40:K40)=4,SUM(H40:K40),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N40" s="13" t="n">
-        <x:f>COUNTIF(D40:K40,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30940,21 +30822,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J41" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K41" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L41" s="14" t="n">
-        <x:f>IF(COUNT(D41:K41)=8,SUM(D41:K41)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M41" s="13" t="n">
-        <x:f>IF(COUNT(H41:K41)=4,SUM(H41:K41),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N41" s="13" t="n">
-        <x:f>COUNTIF(D41:K41,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30993,15 +30872,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L42" s="14" t="n">
-        <x:f>IF(COUNT(D42:K42)=8,SUM(D42:K42)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M42" s="13" t="n">
-        <x:f>IF(COUNT(H42:K42)=4,SUM(H42:K42),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N42" s="13" t="n">
-        <x:f>COUNTIF(D42:K42,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31040,15 +30916,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L43" s="14" t="n">
-        <x:f>IF(COUNT(D43:K43)=8,SUM(D43:K43)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M43" s="13" t="n">
-        <x:f>IF(COUNT(H43:K43)=4,SUM(H43:K43),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N43" s="13" t="n">
-        <x:f>COUNTIF(D43:K43,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31081,21 +30954,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J44" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K44" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L44" s="14" t="n">
-        <x:f>IF(COUNT(D44:K44)=8,SUM(D44:K44)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M44" s="13" t="n">
-        <x:f>IF(COUNT(H44:K44)=4,SUM(H44:K44),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N44" s="13" t="n">
-        <x:f>COUNTIF(D44:K44,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31128,21 +30998,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J45" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K45" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L45" s="14" t="n">
-        <x:f>IF(COUNT(D45:K45)=8,SUM(D45:K45)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M45" s="13" t="n">
-        <x:f>IF(COUNT(H45:K45)=4,SUM(H45:K45),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N45" s="13" t="n">
-        <x:f>COUNTIF(D45:K45,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31175,21 +31042,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J46" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K46" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L46" s="14" t="n">
-        <x:f>IF(COUNT(D46:K46)=8,SUM(D46:K46)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M46" s="13" t="n">
-        <x:f>IF(COUNT(H46:K46)=4,SUM(H46:K46),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N46" s="13" t="n">
-        <x:f>COUNTIF(D46:K46,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31222,21 +31086,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J47" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K47" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L47" s="14" t="n">
-        <x:f>IF(COUNT(D47:K47)=8,SUM(D47:K47)/8,"Pending")</x:f>
-        <x:v>0.875</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M47" s="13" t="n">
-        <x:f>IF(COUNT(H47:K47)=4,SUM(H47:K47),"Pending")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N47" s="13" t="n">
-        <x:f>COUNTIF(D47:K47,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31275,15 +31136,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L48" s="14" t="n">
-        <x:f>IF(COUNT(D48:K48)=8,SUM(D48:K48)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M48" s="13" t="n">
-        <x:f>IF(COUNT(H48:K48)=4,SUM(H48:K48),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N48" s="13" t="n">
-        <x:f>COUNTIF(D48:K48,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31322,15 +31180,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L49" s="14" t="n">
-        <x:f>IF(COUNT(D49:K49)=8,SUM(D49:K49)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M49" s="13" t="n">
-        <x:f>IF(COUNT(H49:K49)=4,SUM(H49:K49),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N49" s="13" t="n">
-        <x:f>COUNTIF(D49:K49,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31363,21 +31218,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J50" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K50" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L50" s="14" t="n">
-        <x:f>IF(COUNT(D50:K50)=8,SUM(D50:K50)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M50" s="13" t="n">
-        <x:f>IF(COUNT(H50:K50)=4,SUM(H50:K50),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N50" s="13" t="n">
-        <x:f>COUNTIF(D50:K50,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31416,15 +31268,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L51" s="14" t="n">
-        <x:f>IF(COUNT(D51:K51)=8,SUM(D51:K51)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M51" s="13" t="n">
-        <x:f>IF(COUNT(H51:K51)=4,SUM(H51:K51),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N51" s="13" t="n">
-        <x:f>COUNTIF(D51:K51,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31463,15 +31312,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L52" s="14" t="n">
-        <x:f>IF(COUNT(D52:K52)=8,SUM(D52:K52)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M52" s="13" t="n">
-        <x:f>IF(COUNT(H52:K52)=4,SUM(H52:K52),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N52" s="13" t="n">
-        <x:f>COUNTIF(D52:K52,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31504,21 +31350,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J53" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K53" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L53" s="14" t="n">
-        <x:f>IF(COUNT(D53:K53)=8,SUM(D53:K53)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M53" s="13" t="n">
-        <x:f>IF(COUNT(H53:K53)=4,SUM(H53:K53),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N53" s="13" t="n">
-        <x:f>COUNTIF(D53:K53,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31551,21 +31394,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J54" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K54" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L54" s="14" t="n">
-        <x:f>IF(COUNT(D54:K54)=8,SUM(D54:K54)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M54" s="13" t="n">
-        <x:f>IF(COUNT(H54:K54)=4,SUM(H54:K54),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N54" s="13" t="n">
-        <x:f>COUNTIF(D54:K54,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31598,21 +31438,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J55" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K55" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L55" s="14" t="n">
-        <x:f>IF(COUNT(D55:K55)=8,SUM(D55:K55)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M55" s="13" t="n">
-        <x:f>IF(COUNT(H55:K55)=4,SUM(H55:K55),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N55" s="13" t="n">
-        <x:f>COUNTIF(D55:K55,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31645,21 +31482,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J56" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K56" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L56" s="14" t="n">
-        <x:f>IF(COUNT(D56:K56)=8,SUM(D56:K56)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M56" s="13" t="n">
-        <x:f>IF(COUNT(H56:K56)=4,SUM(H56:K56),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N56" s="13" t="n">
-        <x:f>COUNTIF(D56:K56,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31692,21 +31526,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J57" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K57" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L57" s="14" t="n">
-        <x:f>IF(COUNT(D57:K57)=8,SUM(D57:K57)/8,"Pending")</x:f>
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M57" s="13" t="n">
-        <x:f>IF(COUNT(H57:K57)=4,SUM(H57:K57),"Pending")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N57" s="13" t="n">
-        <x:f>COUNTIF(D57:K57,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31739,21 +31570,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J58" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K58" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L58" s="14" t="n">
-        <x:f>IF(COUNT(D58:K58)=8,SUM(D58:K58)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M58" s="13" t="n">
-        <x:f>IF(COUNT(H58:K58)=4,SUM(H58:K58),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N58" s="13" t="n">
-        <x:f>COUNTIF(D58:K58,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31786,21 +31614,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J59" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K59" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L59" s="14" t="n">
-        <x:f>IF(COUNT(D59:K59)=8,SUM(D59:K59)/8,"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M59" s="13" t="n">
-        <x:f>IF(COUNT(H59:K59)=4,SUM(H59:K59),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N59" s="13" t="n">
-        <x:f>COUNTIF(D59:K59,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31833,21 +31658,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J60" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K60" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L60" s="14" t="n">
-        <x:f>IF(COUNT(D60:K60)=8,SUM(D60:K60)/8,"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M60" s="13" t="n">
-        <x:f>IF(COUNT(H60:K60)=4,SUM(H60:K60),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N60" s="13" t="n">
-        <x:f>COUNTIF(D60:K60,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31886,15 +31708,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L61" s="14" t="n">
-        <x:f>IF(COUNT(D61:K61)=8,SUM(D61:K61)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M61" s="13" t="n">
-        <x:f>IF(COUNT(H61:K61)=4,SUM(H61:K61),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N61" s="13" t="n">
-        <x:f>COUNTIF(D61:K61,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31927,21 +31746,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J62" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K62" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L62" s="14" t="n">
-        <x:f>IF(COUNT(D62:K62)=8,SUM(D62:K62)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M62" s="13" t="n">
-        <x:f>IF(COUNT(H62:K62)=4,SUM(H62:K62),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N62" s="13" t="n">
-        <x:f>COUNTIF(D62:K62,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -31980,15 +31796,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L63" s="14" t="n">
-        <x:f>IF(COUNT(D63:K63)=8,SUM(D63:K63)/8,"Pending")</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="M63" s="13" t="n">
-        <x:f>IF(COUNT(H63:K63)=4,SUM(H63:K63),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N63" s="13" t="n">
-        <x:f>COUNTIF(D63:K63,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32021,21 +31834,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J64" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K64" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L64" s="14" t="n">
-        <x:f>IF(COUNT(D64:K64)=8,SUM(D64:K64)/8,"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M64" s="13" t="n">
-        <x:f>IF(COUNT(H64:K64)=4,SUM(H64:K64),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N64" s="13" t="n">
-        <x:f>COUNTIF(D64:K64,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32068,21 +31878,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J65" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K65" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L65" s="14" t="n">
-        <x:f>IF(COUNT(D65:K65)=8,SUM(D65:K65)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M65" s="13" t="n">
-        <x:f>IF(COUNT(H65:K65)=4,SUM(H65:K65),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N65" s="13" t="n">
-        <x:f>COUNTIF(D65:K65,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32115,21 +31922,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J66" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K66" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L66" s="14" t="n">
-        <x:f>IF(COUNT(D66:K66)=8,SUM(D66:K66)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M66" s="13" t="n">
-        <x:f>IF(COUNT(H66:K66)=4,SUM(H66:K66),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N66" s="13" t="n">
-        <x:f>COUNTIF(D66:K66,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32168,15 +31972,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L67" s="14" t="n">
-        <x:f>IF(COUNT(D67:K67)=8,SUM(D67:K67)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M67" s="13" t="n">
-        <x:f>IF(COUNT(H67:K67)=4,SUM(H67:K67),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N67" s="13" t="n">
-        <x:f>COUNTIF(D67:K67,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32209,21 +32010,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J68" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K68" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L68" s="14" t="n">
-        <x:f>IF(COUNT(D68:K68)=8,SUM(D68:K68)/8,"Pending")</x:f>
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M68" s="13" t="n">
-        <x:f>IF(COUNT(H68:K68)=4,SUM(H68:K68),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N68" s="13" t="n">
-        <x:f>COUNTIF(D68:K68,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32262,15 +32060,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L69" s="14" t="n">
-        <x:f>IF(COUNT(D69:K69)=8,SUM(D69:K69)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M69" s="13" t="n">
-        <x:f>IF(COUNT(H69:K69)=4,SUM(H69:K69),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N69" s="13" t="n">
-        <x:f>COUNTIF(D69:K69,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32309,15 +32104,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L70" s="14" t="n">
-        <x:f>IF(COUNT(D70:K70)=8,SUM(D70:K70)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M70" s="13" t="n">
-        <x:f>IF(COUNT(H70:K70)=4,SUM(H70:K70),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N70" s="13" t="n">
-        <x:f>COUNTIF(D70:K70,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32350,21 +32142,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J71" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K71" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L71" s="14" t="n">
-        <x:f>IF(COUNT(D71:K71)=8,SUM(D71:K71)/8,"Pending")</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M71" s="13" t="n">
-        <x:f>IF(COUNT(H71:K71)=4,SUM(H71:K71),"Pending")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N71" s="13" t="n">
-        <x:f>COUNTIF(D71:K71,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32403,15 +32192,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L72" s="14" t="n">
-        <x:f>IF(COUNT(D72:K72)=8,SUM(D72:K72)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M72" s="13" t="n">
-        <x:f>IF(COUNT(H72:K72)=4,SUM(H72:K72),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N72" s="13" t="n">
-        <x:f>COUNTIF(D72:K72,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32450,15 +32236,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L73" s="14" t="n">
-        <x:f>IF(COUNT(D73:K73)=8,SUM(D73:K73)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M73" s="13" t="n">
-        <x:f>IF(COUNT(H73:K73)=4,SUM(H73:K73),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N73" s="13" t="n">
-        <x:f>COUNTIF(D73:K73,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32491,21 +32274,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J74" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K74" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L74" s="14" t="n">
-        <x:f>IF(COUNT(D74:K74)=8,SUM(D74:K74)/8,"Pending")</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M74" s="13" t="n">
-        <x:f>IF(COUNT(H74:K74)=4,SUM(H74:K74),"Pending")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N74" s="13" t="n">
-        <x:f>COUNTIF(D74:K74,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32544,15 +32324,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L75" s="14" t="n">
-        <x:f>IF(COUNT(D75:K75)=8,SUM(D75:K75)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M75" s="13" t="n">
-        <x:f>IF(COUNT(H75:K75)=4,SUM(H75:K75),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N75" s="13" t="n">
-        <x:f>COUNTIF(D75:K75,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32591,15 +32368,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L76" s="14" t="n">
-        <x:f>IF(COUNT(D76:K76)=8,SUM(D76:K76)/8,"Pending")</x:f>
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="M76" s="13" t="n">
-        <x:f>IF(COUNT(H76:K76)=4,SUM(H76:K76),"Pending")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N76" s="13" t="n">
-        <x:f>COUNTIF(D76:K76,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -32638,15 +32412,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L77" s="14" t="n">
-        <x:f>IF(COUNT(D77:K77)=8,SUM(D77:K77)/8,"Pending")</x:f>
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="M77" s="13" t="n">
-        <x:f>IF(COUNT(H77:K77)=4,SUM(H77:K77),"Pending")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="N77" s="13" t="n">
-        <x:f>COUNTIF(D77:K77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -35668,11 +35439,11 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>COUNTIF('Study REB Profile'!J2:J77,1)</x:f>
-        <x:v>19</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>B8/76</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.3815789473684211</x:v>
       </x:c>
       <x:c r="D8" s="13" t="n">
         <x:f>COUNTIF('Study REB Profile'!J2:J77,"U")</x:f>
@@ -35760,7 +35531,7 @@
       </x:c>
       <x:c r="B13" s="14" t="n">
         <x:f>AVERAGE('Study REB Profile'!L2:L77)</x:f>
-        <x:v>0.6398026315789473</x:v>
+        <x:v>0.65625</x:v>
       </x:c>
       <x:c r="C13" s="12"/>
       <x:c r="D13" s="12"/>

</xml_diff>

<commit_message>
Synchronize corrected L7 consensus ratings
</commit_message>
<xml_diff>
--- a/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
+++ b/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R154999075af64e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R8e3be05f19484ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb705d1291f0b49ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R94f707ed863b4e4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="Rec1cc6967a2944ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Rf21b7ac4ca5e49d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="R758dee57a6ec4ec6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R81109aaaeaa24588"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="Ra07359923a6f4c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Rdf72f128c62f42d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="Rd244073ab7794344"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Rbe37bb6646f14035"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R6de5bbe6404f43b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rba3fbdf31a744d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="Rbbd0730fa0ad4579"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Recbfc27fa4244023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="Rd0cfec9df75a44f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="Re001d9855fe3499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R5efd07df9a9c41a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5181c451aa8a40d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R16d1eff36c7d4f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb20a4e0399af4464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R4ebc4b0db83545c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="R9cf9c1a4231d4152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Rb8d3fb0501074c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="R1ea4bdab68944a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R4f2497922b114e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="R934dd511b4a0471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Ra781194e57ca4971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="R1f0430fdb9e44f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Raacae2bfa7394fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R452ae651b6084fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Ra4b15a5c701e4f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="R87b1a01e702a4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="R238275a0779d44a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R50df982993af4caa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R4640b4caff464e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R2b24428a42c042dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5057,10 +5057,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C200" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D200" s="12" t="str">
-        <x:v>Skin temperature underneath the taped probe was quantified during use, providing an interface-safety endpoint.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E200" s="12" t="str">
         <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
@@ -5069,7 +5069,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G200" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="15" hidden="0" customHeight="1">
@@ -7449,10 +7449,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C304" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D304" s="12" t="str">
-        <x:v>The assembled supports were quantitatively validated in the wearable robot.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E304" s="12" t="str">
         <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
@@ -7461,7 +7461,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G304" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="305" ht="15" hidden="0" customHeight="1">
@@ -7633,10 +7633,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C312" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D312" s="12" t="str">
-        <x:v>The complete earable was tested on a person during rest and cycling.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E312" s="12" t="str">
         <x:v>PDF pp. 2–7; Figs. 1–5</x:v>
@@ -7645,7 +7645,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G312" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="313" ht="15" hidden="0" customHeight="1">
@@ -8001,10 +8001,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C328" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D328" s="12" t="str">
-        <x:v>The sensor was attached to the body for multiple quantitative demonstrations.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E328" s="12" t="str">
         <x:v>PDF pp. 3–13; Figs. 1–9</x:v>
@@ -8013,7 +8013,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G328" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="329" ht="15" hidden="0" customHeight="1">
@@ -9105,10 +9105,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C376" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D376" s="12" t="str">
-        <x:v>The complete wearable was evaluated in five volunteers against BioHarness.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E376" s="12" t="str">
         <x:v>PDF pp. 3–15; Figs. 1–9; cited Supplementary Table S1</x:v>
@@ -9117,7 +9117,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G376" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Rule-clarification recode</x:v>
       </x:c>
     </x:row>
     <x:row r="377" ht="24" hidden="0" customHeight="1">
@@ -9289,10 +9289,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C384" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D384" s="12" t="str">
-        <x:v>Four sensors were integrated into a shoe and produced quantitative resistance traces.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E384" s="12" t="str">
         <x:v>PDF pp. 2–15; Figs. 1–10; Tables 1–4</x:v>
@@ -9301,7 +9301,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G384" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="385" ht="15" hidden="0" customHeight="1">
@@ -9657,10 +9657,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C400" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D400" s="12" t="str">
-        <x:v>The sensor was placed beneath the foot and recorded walking/running signals.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E400" s="12" t="str">
         <x:v>PDF pp. 2–12; Figs. 1–9; Tables 1–2</x:v>
@@ -9669,7 +9669,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G400" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Rule-clarification recode</x:v>
       </x:c>
     </x:row>
     <x:row r="401" ht="15" hidden="0" customHeight="1">
@@ -9841,10 +9841,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C408" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D408" s="12" t="str">
-        <x:v>Embedded sensors were quantitatively demonstrated in helmet, finger and soft structures.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E408" s="12" t="str">
         <x:v>PDF pp. 2–12; Figs. 1–10; Table 1</x:v>
@@ -9853,7 +9853,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G408" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="409" ht="15" hidden="0" customHeight="1">
@@ -11497,10 +11497,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C480" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D480" s="12" t="str">
-        <x:v>The complete device was tested on eight participants against a commercial reference.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E480" s="12" t="str">
         <x:v>PDF pp. 3–9; Figs. 1–13</x:v>
@@ -11509,7 +11509,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G480" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="481" ht="15" hidden="0" customHeight="1">
@@ -11865,10 +11865,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C496" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D496" s="12" t="str">
-        <x:v>The complete nanogenerator was demonstrated for touch, mouse clicks and finger-joint motion.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E496" s="12" t="str">
         <x:v>PDF pp. 3–8; Figs. 1–6; cited Supplementary Figs. S1–S10</x:v>
@@ -11877,7 +11877,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G496" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>Rule-clarification recode</x:v>
       </x:c>
     </x:row>
     <x:row r="497" ht="24" hidden="0" customHeight="1">
@@ -12601,10 +12601,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C528" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D528" s="12" t="str">
-        <x:v>Completed sensors generated respiration and gait signals after body placement.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E528" s="12" t="str">
         <x:v>PDF pp. 2, 4–12; Figs. 1–8</x:v>
@@ -12613,7 +12613,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G528" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="529" ht="24" hidden="0" customHeight="1">
@@ -12969,10 +12969,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C544" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D544" s="12" t="str">
-        <x:v>The completed fibre sensor produced repeated signals at several body sites and in tactile tests.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E544" s="12" t="str">
         <x:v>PDF pp. 4–12; Figs. 1–7; Supplementary Figs. S1–S5 cited</x:v>
@@ -12981,7 +12981,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G544" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="545" ht="24" hidden="0" customHeight="1">
@@ -13153,10 +13153,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C552" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D552" s="12" t="str">
-        <x:v>Completed sensors generated quantitative human-motion, tactile and matrix signals.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E552" s="12" t="str">
         <x:v>PDF pp. 4–11; Figs. 1–8; Supplementary Figs. S1–S5 cited</x:v>
@@ -13165,7 +13165,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G552" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="553" ht="24" hidden="0" customHeight="1">
@@ -13521,10 +13521,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C568" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D568" s="12" t="str">
-        <x:v>The completed sensor generated repeated facial, throat, speech and finger signals.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E568" s="12" t="str">
         <x:v>PDF pp. 2–9; Figs. 1–6; Supporting Figs. S1–S3 and Table S1 cited</x:v>
@@ -13533,7 +13533,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G568" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Rule-clarification recode</x:v>
       </x:c>
     </x:row>
     <x:row r="569" ht="24" hidden="0" customHeight="1">
@@ -13705,10 +13705,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C576" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D576" s="12" t="str">
-        <x:v>The completed sensor generated repeated human-motion signals.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E576" s="12" t="str">
         <x:v>PDF pp. 2–7; Figs. 1–5; Supplementary Figs. S1–S7 cited</x:v>
@@ -13717,7 +13717,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G576" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Rule-clarification recode</x:v>
       </x:c>
     </x:row>
     <x:row r="577" ht="24" hidden="0" customHeight="1">
@@ -14073,10 +14073,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C592" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D592" s="12" t="str">
-        <x:v>The completed sensor generated repeated signals from several body motions and physiological activities.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E592" s="12" t="str">
         <x:v>PDF pp. 10–35 of available accepted manuscript; Figs. 1–10; Tables 1–2; Supplementary Tables S1–S2 cited</x:v>
@@ -14085,7 +14085,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G592" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="593" ht="36" hidden="0" customHeight="1">
@@ -14441,10 +14441,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C608" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D608" s="12" t="str">
-        <x:v>The complete strip-and-contact measurement assembly is tested repeatedly and retained function is described across 25 sensing cycles.</x:v>
+        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
       </x:c>
       <x:c r="E608" s="12" t="str">
         <x:v>PDF pp. 1–8; Figs. 2, 6–11; Table 1; ESI Table S1 and Fig. S5 cited</x:v>
@@ -14453,7 +14453,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G608" s="12" t="str">
-        <x:v>Batch 09</x:v>
+        <x:v>Adjudicated to Reviewer 2</x:v>
       </x:c>
     </x:row>
     <x:row r="609" ht="24" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Reconcile L7 consensus classifications
</commit_message>
<xml_diff>
--- a/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
+++ b/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5181c451aa8a40d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R16d1eff36c7d4f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb20a4e0399af4464"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R4ebc4b0db83545c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="R9cf9c1a4231d4152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Rb8d3fb0501074c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="R1ea4bdab68944a15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R4f2497922b114e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="R934dd511b4a0471a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Ra781194e57ca4971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="R1f0430fdb9e44f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Raacae2bfa7394fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R452ae651b6084fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Ra4b15a5c701e4f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="R87b1a01e702a4873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="R238275a0779d44a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R50df982993af4caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R4640b4caff464e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R2b24428a42c042dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rba012b6e3f4247af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R6d34eeb97bf4481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb6288531edf54367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R3e65555e28aa49d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="R8ee214fdfb9448d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Ref212166c5954855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="Racdcd1782a134081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R010e7183140e44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="R9b28380804bd4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Rcb363ef7bb7341c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="Rd974bc0fbf3d4b4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Re40a743cc35d48df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R2c403d0a5a09488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rfdef40847538455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="Rbe614843c17d4339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Re437d45c411d497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R27fbd55db8b54216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R77fc1e83dcf54c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="Rfd43a54c4d574780"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -447,7 +447,7 @@
         <x:v>Consensus provenance</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>The final profiles use the finalized L7 decisions in Supplementary Data 4. Article-specific reasons and locators are retained in REB Coding.</x:v>
+        <x:v>The final profiles use the complete two-route L7 audit recorded in Supplementary Data 4. Article-specific reasons and locators are retained in REB Coding.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -641,19 +641,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>The authors assess GRF pattern and stance-phase repeatability throughout sequential worn gait cycles and discuss biological variability. This is direct qualitative cross-cycle evaluation, not a retention percentage.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
         <x:v>S001_Main.pdf, physical p. 7 protocol; pp. 13-15, Fig. 7a-b and sequential-gait repeatability discussion.</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -834,10 +834,10 @@
         <x:v>PDF pp. 1-13 and Supplement checked</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1009,19 +1009,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C24" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Section 3.3 reports repeatable resistance changes during repeated hand/finger actions with attached sensors. Qualification does not depend on the separate bench durability or stepping demonstration.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
         <x:v>S004_Main.pdf, physical pp. 11-12, section 3.3/Fig. 7a-e.</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1202,10 +1202,10 @@
         <x:v>PDF pp. 3–11; Figs. 1–9; Tables 1–3</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -1386,10 +1386,10 @@
         <x:v>S007_Main.pdf, physical pp. 10-11, section 3.2, Figs. 9-10 and Table 3; on-person sections pp. 7-9.</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G40" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -1573,7 +1573,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G48" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -1754,10 +1754,10 @@
         <x:v>PDF pp. 3–16; Figs. 1–13; Appendix A</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G56" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
@@ -1941,7 +1941,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G64" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
@@ -2125,7 +2125,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G72" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -2306,10 +2306,10 @@
         <x:v>PDF pp. 3–7; Figs. 1–6; Table 1; cited SI</x:v>
       </x:c>
       <x:c r="F80" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G80" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
@@ -2484,16 +2484,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D88" s="12" t="str">
-        <x:v>Three pull-out specimens per material and &gt;12 N interface outcome.</x:v>
+        <x:v>Route A—direct interface: three pull-out specimens per material quantified the fibre–printed-host interface, with pull-out force exceeding 12 N without complete detachment.</x:v>
       </x:c>
       <x:c r="E88" s="12" t="str">
         <x:v>PDF pp. 4–15; Figs. 1–10; Tables 1–2</x:v>
       </x:c>
       <x:c r="F88" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G88" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
@@ -2674,10 +2674,10 @@
         <x:v>PDF pp. 3–11; Figs. 1–6; Table 1</x:v>
       </x:c>
       <x:c r="F96" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G96" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="15" hidden="0" customHeight="1">
@@ -2858,10 +2858,10 @@
         <x:v>PDF pp. 3-5 checked</x:v>
       </x:c>
       <x:c r="F104" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G104" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="15" hidden="0" customHeight="1">
@@ -3036,16 +3036,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D112" s="12" t="str">
-        <x:v>Hundreds of loaded steps were completed and the insole was reported airtight and intact.</x:v>
+        <x:v>Route B—integrated assembly: the final insole completed repeated loaded steps and the pneumatic chambers remained airtight and intact throughout the reported loading sequence.</x:v>
       </x:c>
       <x:c r="E112" s="12" t="str">
         <x:v>PDF pp. 3–11; Figs. 1–6; Table 1</x:v>
       </x:c>
       <x:c r="F112" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G112" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="15" hidden="0" customHeight="1">
@@ -3226,10 +3226,10 @@
         <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
       </x:c>
       <x:c r="F120" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G120" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="15" hidden="0" customHeight="1">
@@ -3413,7 +3413,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G128" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15" hidden="0" customHeight="1">
@@ -3588,16 +3588,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D136" s="12" t="str">
-        <x:v>Removal/re-wearing and a separate-session validation quantify integrated-system transfer after reapplication.</x:v>
+        <x:v>Route B—integrated assembly: the data glove was removed and re-worn for a separate-session validation, with retained classification performance reported after reapplication.</x:v>
       </x:c>
       <x:c r="E136" s="12" t="str">
         <x:v>PDF pp. 3–12; Figs. 1–8; Table 1</x:v>
       </x:c>
       <x:c r="F136" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G136" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="15" hidden="0" customHeight="1">
@@ -3769,19 +3769,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C144" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D144" s="12" t="str">
-        <x:v>Normal walking produces periodic waveforms with uniform amplitude, contrasted with variable limping signals; the sole configuration is shown alongside the worn application.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E144" s="12" t="str">
         <x:v>S022_Main.pdf, physical p. 6, full-body monitoring paragraph; p. 7, Fig. 6h-j. Supplied supplement contains separate bench characterization.</x:v>
       </x:c>
       <x:c r="F144" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G144" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="15" hidden="0" customHeight="1">
@@ -3962,10 +3962,10 @@
         <x:v>PDF pp. 3–16; Figs. 2–10; Tables 1–2</x:v>
       </x:c>
       <x:c r="F152" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G152" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="15" hidden="0" customHeight="1">
@@ -4140,16 +4140,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D160" s="12" t="str">
-        <x:v>Lap-shear adhesion provides a quantitative encapsulation-interface endpoint.</x:v>
+        <x:v>Route A—direct interface: lap-shear testing quantified adhesion between the conductive TPU layer and the pressure-sensitive adhesive encapsulation.</x:v>
       </x:c>
       <x:c r="E160" s="12" t="str">
         <x:v>PDF pp. 2–11; Figs. 1–6; cited SI</x:v>
       </x:c>
       <x:c r="F160" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G160" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
@@ -4333,7 +4333,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G168" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
@@ -4514,10 +4514,10 @@
         <x:v>PDF pp. 4–17; Figs. 1–10; Tables 1–4</x:v>
       </x:c>
       <x:c r="F176" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G176" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
@@ -4701,7 +4701,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G184" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="15" hidden="0" customHeight="1">
@@ -4882,10 +4882,10 @@
         <x:v>PDF pp. 3–12; Figs. 1–9; Tables 1–3; Appendix A</x:v>
       </x:c>
       <x:c r="F192" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G192" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="24" hidden="0" customHeight="1">
@@ -5066,10 +5066,10 @@
         <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
       </x:c>
       <x:c r="F200" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G200" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="15" hidden="0" customHeight="1">
@@ -5241,19 +5241,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C208" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D208" s="12" t="str">
-        <x:v>The 1000-cycle experiment reports about 30% initial resistance reduction under specimen pressure loading. Fig. 5 demonstrates body-motion response.</x:v>
+        <x:v>Route A—direct interface: peel-off force was measured for coated, embedded and unmodified TPE sensing units pressed against test tape, directly evaluating retention of the CNT–TPE sensing interface.</x:v>
       </x:c>
       <x:c r="E208" s="12" t="str">
-        <x:v>S033_Main.pdf, physical pp. 5-7, Figs. 4e and 5; S033_Supplement_01.pdf, pp. 2-3/Figs. S1-S4; supplied Videos S1-S2.</x:v>
+        <x:v>S033_Supplement_01.pdf, p. 2, Fig. S2; S033_Main.pdf, physical pp. 5–7</x:v>
       </x:c>
       <x:c r="F208" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G208" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="15" hidden="0" customHeight="1">
@@ -5425,19 +5425,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C216" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D216" s="12" t="str">
-        <x:v>The authors report no carryover after rinsing. Sweat collection/contact is demonstrated, but the rinse/reuse experiments do not establish a repeatedly attached body-worn assembly.</x:v>
+        <x:v>Route A—direct interface: leakage was monitored during repeated wash/reuse cycles of the fused microfluidic-on-fabric structure; fabric devices remained functional for 60–70 cycles and the complete platform retained stable voltage readings over 30 reuse cycles.</x:v>
       </x:c>
       <x:c r="E216" s="12" t="str">
-        <x:v>S034_Main.pdf, physical pp. 8-10, biofluid applications, reuse discussion and Conclusions.</x:v>
+        <x:v>S034_Main.pdf, physical pp. 4–7, Figs. 1C and 3B–D</x:v>
       </x:c>
       <x:c r="F216" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G216" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="15" hidden="0" customHeight="1">
@@ -5621,7 +5621,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G224" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="15" hidden="0" customHeight="1">
@@ -5796,16 +5796,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D232" s="12" t="str">
-        <x:v>The attached sweat-rate device cannot accommodate the entire exercise's perspiration volume; monitoring ends at approximately 2200 seconds because its capacity is insufficient.</x:v>
+        <x:v>Route B—integrated assembly: the attached sweat-rate device was monitored until the explicit system-capacity failure endpoint at approximately 2200 seconds.</x:v>
       </x:c>
       <x:c r="E232" s="12" t="str">
-        <x:v>S036_Main.pdf, physical p. 3, assembly/cycling protocol; pp. 9-10, on-body section, p. 10 first paragraph/Fig. 6.</x:v>
+        <x:v>S036_Main.pdf, physical p. 3, assembly/cycling protocol; pp. 9–10, on-body section and Fig. 6</x:v>
       </x:c>
       <x:c r="F232" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G232" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="233" ht="15" hidden="0" customHeight="1">
@@ -5986,10 +5986,10 @@
         <x:v>PDF pp. 1–10; Figs. 1–16</x:v>
       </x:c>
       <x:c r="F240" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G240" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="241" ht="15" hidden="0" customHeight="1">
@@ -6161,19 +6161,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C248" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D248" s="12" t="str">
-        <x:v>The text explicitly reports relatively repeatable resistance responses across all three flexing cycles at the specified positions.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E248" s="12" t="str">
         <x:v>S038_Main.pdf, physical p. 12, section 3.5 and Fig. 11b-c.</x:v>
       </x:c>
       <x:c r="F248" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G248" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="15" hidden="0" customHeight="1">
@@ -6345,19 +6345,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C256" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D256" s="12" t="str">
-        <x:v>The printed finger glove returned to its initial signal during continuous bending/releasing motions.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E256" s="12" t="str">
         <x:v>PDF pp. 3–9; Figs. 2–10</x:v>
       </x:c>
       <x:c r="F256" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G256" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="257" ht="15" hidden="0" customHeight="1">
@@ -6538,10 +6538,10 @@
         <x:v>PDF pp. 2–12; Figs. 1–8; Tables 1–4; cited SI</x:v>
       </x:c>
       <x:c r="F264" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G264" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="265" ht="15" hidden="0" customHeight="1">
@@ -6722,10 +6722,10 @@
         <x:v>PDF pp. 4–11; Figs. 1, 5–6; cited SI</x:v>
       </x:c>
       <x:c r="F272" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G272" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="273" ht="15" hidden="0" customHeight="1">
@@ -6897,19 +6897,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C280" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D280" s="12" t="str">
-        <x:v>A Z-shaped spring embedded in the author's insole is assessed during repeated walking at two frequencies; maintained stable voltage is explicitly reported.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E280" s="12" t="str">
         <x:v>S046_Main.pdf, physical pp. 6-7, Fig. 5c-e and application paragraph (printed pp. 1021-1022).</x:v>
       </x:c>
       <x:c r="F280" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G280" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="281" ht="24" hidden="0" customHeight="1">
@@ -7084,16 +7084,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D288" s="12" t="str">
-        <x:v>Pressure is recorded to confirm maintenance of 15-25 mmHg; section 3.2.1 reports that mean pressure is maintained through the trial with strap adjustment.</x:v>
+        <x:v>Route B—integrated assembly: interface pressure was monitored during the wear trial and maintained within the stated 15–25 mmHg range, with strap adjustment recorded.</x:v>
       </x:c>
       <x:c r="E288" s="12" t="str">
-        <x:v>S047_Main.pdf, physical p. 6, clinical protocol; pp. 9-10, section 3.2.1/Fig. 9. The figure shows the initial hour; adjacent text reports trial-period maintenance.</x:v>
+        <x:v>S047_Main.pdf, physical p. 6, clinical protocol; pp. 9–10, section 3.2.1 and Fig. 9</x:v>
       </x:c>
       <x:c r="F288" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G288" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="289" ht="15" hidden="0" customHeight="1">
@@ -7265,19 +7265,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C296" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D296" s="12" t="str">
-        <x:v>Body-mounted demonstrations were reported without a quantitative interface or pre/post integration endpoint.</x:v>
+        <x:v>Route A—direct interface: surface- and interface-embedded graphene/TPU samples underwent four hours of solvent ultrasonication with resistance monitoring and inspection for delamination, shedding, swelling and retained graphene at the interface.</x:v>
       </x:c>
       <x:c r="E296" s="12" t="str">
-        <x:v>PDF pp. 3–9; Figs. 1, 4–9; cited SI</x:v>
+        <x:v>S048_Main.pdf, physical pp. 3–6, Fig. 4; Supplementary Figs. S7–S8</x:v>
       </x:c>
       <x:c r="F296" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G296" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="297" ht="15" hidden="0" customHeight="1">
@@ -7458,10 +7458,10 @@
         <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
       </x:c>
       <x:c r="F304" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G304" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="305" ht="15" hidden="0" customHeight="1">
@@ -7642,10 +7642,10 @@
         <x:v>PDF pp. 2–7; Figs. 1–5</x:v>
       </x:c>
       <x:c r="F312" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G312" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="313" ht="15" hidden="0" customHeight="1">
@@ -7817,19 +7817,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C320" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D320" s="12" t="str">
-        <x:v>The final hand-worn sensor was quantitatively evaluated across five object-manipulation classes.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E320" s="12" t="str">
         <x:v>PDF pp. 10-12; Fig. 6</x:v>
       </x:c>
       <x:c r="F320" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G320" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="321" ht="24" hidden="0" customHeight="1">
@@ -8010,10 +8010,10 @@
         <x:v>PDF pp. 3–13; Figs. 1–9</x:v>
       </x:c>
       <x:c r="F328" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G328" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="329" ht="15" hidden="0" customHeight="1">
@@ -8194,10 +8194,10 @@
         <x:v>PDF pp. 3–9; Figs. 1–7; Appendix 1</x:v>
       </x:c>
       <x:c r="F336" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G336" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="337" ht="15" hidden="0" customHeight="1">
@@ -8369,19 +8369,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C344" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D344" s="12" t="str">
-        <x:v>After initial gait adjustment, the body-attached sensor gives a consistent walking output over the reported 10-second interval. Separate 11600-cycle compression is not used for this score.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E344" s="12" t="str">
         <x:v>S055_Main.pdf, physical p. 7, section 2.6; p. 9, Fig. 6a. Fig. 5g concerns bench durability.</x:v>
       </x:c>
       <x:c r="F344" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G344" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="345" ht="15" hidden="0" customHeight="1">
@@ -8553,19 +8553,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C352" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D352" s="12" t="str">
-        <x:v>The authors evaluate stable signal patterns for repeated calf/neck/larynx actions and stable responses for repeated joint movements in the worn demonstrations.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E352" s="12" t="str">
         <x:v>S056_Main.pdf, physical p. 13, Fig. 11a-h; p. 14, accompanying interpretation and Fig. 12b-c.</x:v>
       </x:c>
       <x:c r="F352" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G352" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="353" ht="15" hidden="0" customHeight="1">
@@ -8737,19 +8737,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C360" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D360" s="12" t="str">
-        <x:v>Attached throat sensors produce distinct, reproducible swallowing/coughing profiles; the finger/wrist trials also receive an explicit repeatability assessment.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E360" s="12" t="str">
         <x:v>S057_Main.pdf, physical pp. 15-16, section 3.3/Fig. 15c-e, especially p. 16 opening paragraph.</x:v>
       </x:c>
       <x:c r="F360" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G360" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="361" ht="15" hidden="0" customHeight="1">
@@ -8924,16 +8924,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D368" s="12" t="str">
-        <x:v>Supplementary Fig. S7c explicitly documents seven days of wear. The paper reports no structural damage, delamination or output failure after the reliability evaluation.</x:v>
+        <x:v>Route B—integrated assembly: a seven-day wear trial was documented and the reliability assessment reported no structural damage, delamination or output failure.</x:v>
       </x:c>
       <x:c r="E368" s="12" t="str">
-        <x:v>S058_Supplement_01.docx, Fig. S7c (7-day wear trial); S058_Main.pdf, physical p. 8, reliability discussion, and p. 12, methods.</x:v>
+        <x:v>S058_Supplement_01.docx, Fig. S7c; S058_Main.pdf, physical pp. 8 and 12</x:v>
       </x:c>
       <x:c r="F368" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G368" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="369" ht="24" hidden="0" customHeight="1">
@@ -9105,19 +9105,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C376" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D376" s="12" t="str">
-        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
+        <x:v>Route B—integrated assembly: the encapsulated Int1 configuration completed 1000 loading cycles with continuous output, no spikes, signal loss or visible mechanical damage; baseline drift and retained structural integrity were explicitly reported.</x:v>
       </x:c>
       <x:c r="E376" s="12" t="str">
-        <x:v>PDF pp. 3–15; Figs. 1–9; cited Supplementary Table S1</x:v>
+        <x:v>S059_Main.pdf, physical pp. 7–8, Fig. 3C</x:v>
       </x:c>
       <x:c r="F376" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G376" s="12" t="str">
-        <x:v>Rule-clarification recode</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="377" ht="24" hidden="0" customHeight="1">
@@ -9298,10 +9298,10 @@
         <x:v>PDF pp. 2–15; Figs. 1–10; Tables 1–4</x:v>
       </x:c>
       <x:c r="F384" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G384" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="385" ht="15" hidden="0" customHeight="1">
@@ -9485,7 +9485,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G392" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="393" ht="15" hidden="0" customHeight="1">
@@ -9666,10 +9666,10 @@
         <x:v>PDF pp. 2–12; Figs. 1–9; Tables 1–2</x:v>
       </x:c>
       <x:c r="F400" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G400" s="12" t="str">
-        <x:v>Rule-clarification recode</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="401" ht="15" hidden="0" customHeight="1">
@@ -9841,19 +9841,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C408" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D408" s="12" t="str">
-        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
+        <x:v>Route A—direct integration: repeated impact testing compared surface-mounted and embedded sensors; the surface-mounted layer crushed, fragmented and peeled, whereas the embedded sensor survived and retained functional stability.</x:v>
       </x:c>
       <x:c r="E408" s="12" t="str">
-        <x:v>PDF pp. 2–12; Figs. 1–10; Table 1</x:v>
+        <x:v>S064_Main.pdf, physical pp. 6–8, Figs. 4–6</x:v>
       </x:c>
       <x:c r="F408" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G408" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="409" ht="15" hidden="0" customHeight="1">
@@ -10028,16 +10028,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D416" s="12" t="str">
-        <x:v>The authors explicitly evaluate durability during repeated bending and report no delamination or loss of sensitivity, with consistent cycle responses and SNR 34.12 ± 0.72.</x:v>
+        <x:v>Route B—integrated assembly: repeated attached-sensor bending was evaluated with no delamination or loss of sensitivity, consistent cycle responses and SNR of 34.12 ± 0.72.</x:v>
       </x:c>
       <x:c r="E416" s="12" t="str">
-        <x:v>S065_Main.pdf, physical pp. 8-9, section 3.4/Fig. 7c-d.</x:v>
+        <x:v>S065_Main.pdf, physical pp. 8–9, section 3.4 and Fig. 7c–d</x:v>
       </x:c>
       <x:c r="F416" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G416" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="417" ht="15" hidden="0" customHeight="1">
@@ -10212,16 +10212,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D424" s="12" t="str">
-        <x:v>The long-term monitoring section explicitly reports stable amplitude, no drift and no lost periodicity across the recording.</x:v>
+        <x:v>Route B—integrated assembly: the complete chest-strap system was monitored for approximately 42 minutes; stable amplitude, no evident drift and no loss of periodicity were reported.</x:v>
       </x:c>
       <x:c r="E424" s="12" t="str">
-        <x:v>S066_Main.pdf, physical p. 5, assembly; pp. 7-8, section V.C, Long-Term Monitoring/Fig. 6.</x:v>
+        <x:v>S066_Main.pdf, physical p. 5, assembly; pp. 7–8, section V.C and Fig. 6</x:v>
       </x:c>
       <x:c r="F424" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G424" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="425" ht="15" hidden="0" customHeight="1">
@@ -10393,19 +10393,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C432" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D432" s="12" t="str">
-        <x:v>Absolute amplitudes fluctuate, but the text explicitly reports preserved periodicity, inter-peak timing and relative peak relationships across environmental conditions.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E432" s="12" t="str">
         <x:v>S067_Main.pdf, physical pp. 7-9, Fig. 4e-f and environmental robustness discussion referring to Fig. S6.</x:v>
       </x:c>
       <x:c r="F432" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G432" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="433" ht="15" hidden="0" customHeight="1">
@@ -10577,19 +10577,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C440" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D440" s="12" t="str">
-        <x:v>The wrist-mounted sensor is assessed during repeated moderate-force closures; authors describe the waveform as repeatable, with consistent swallowing response in the separate throat configuration.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E440" s="12" t="str">
         <x:v>S068_Main.pdf, physical pp. 8-9, section 3.8/Fig. 7c,e.</x:v>
       </x:c>
       <x:c r="F440" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G440" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="441" ht="15" hidden="0" customHeight="1">
@@ -10761,19 +10761,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C448" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D448" s="12" t="str">
-        <x:v>20000 cycles, detergent washing and peel testing assess material/device durability off-body. Supplied video samples show chamber tests, LEDs and table-top finger contact.</x:v>
+        <x:v>Route A—direct interface: the printed-polypropylene/conductive-fabric bond was evaluated using the DIN EN ISO 11339 T-peel method. The study also reported stable output over 20,000 cycles and no delamination during repeated operation.</x:v>
       </x:c>
       <x:c r="E448" s="12" t="str">
-        <x:v>S069_Main.pdf, physical pp. 11-13, Figs. 10f-g/11; S069_Supplement_01.docx and Supplements 02-04 videos.</x:v>
+        <x:v>S069_Main.pdf, physical pp. 11–13, Fig. 10f–g; Supplementary Fig. S11</x:v>
       </x:c>
       <x:c r="F448" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G448" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="449" ht="15" hidden="0" customHeight="1">
@@ -10945,19 +10945,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C456" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D456" s="12" t="str">
-        <x:v>The conclusion explicitly reports stable and repeatable response during controlled wearable movement cycles; section V defines the worn protocol.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E456" s="12" t="str">
         <x:v>S070_Main.pdf, physical p. 8, section V; p. 9, Fig. 9; p. 10, wearable-validation conclusion.</x:v>
       </x:c>
       <x:c r="F456" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G456" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="457" ht="15" hidden="0" customHeight="1">
@@ -11132,16 +11132,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D464" s="12" t="str">
-        <x:v>Ten gait cycles per test are analyzed at slow/fast speeds; the authors expressly evaluate stability and reproducibility of the worn sensor across these motion trials.</x:v>
+        <x:v>Route A—direct interface: after 1000 compression cycles, coating integrity was inspected by SEM; the graphene layer remained attached to the TPU substrate without large-scale delamination, peeling or shedding.</x:v>
       </x:c>
       <x:c r="E464" s="12" t="str">
-        <x:v>S071_Main.pdf, physical pp. 9-10, section 3.3/Figs. 11-12.</x:v>
+        <x:v>S071_Main.pdf, physical pp. 5–6, Fig. 6f–g</x:v>
       </x:c>
       <x:c r="F464" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G464" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="465" ht="15" hidden="0" customHeight="1">
@@ -11313,19 +11313,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C472" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D472" s="12" t="str">
-        <x:v>During worn nominal-angle flexion cycles, peak/interval variability is acknowledged and its effect on the repeated signal trend is evaluated. The response is not claimed to be perfectly repeatable.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E472" s="12" t="str">
         <x:v>S073_Main.pdf, physical pp. 7-8, section 3.2/Fig. 7, especially p. 8 first two paragraphs.</x:v>
       </x:c>
       <x:c r="F472" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G472" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="473" ht="15" hidden="0" customHeight="1">
@@ -11506,10 +11506,10 @@
         <x:v>PDF pp. 3–9; Figs. 1–13</x:v>
       </x:c>
       <x:c r="F480" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G480" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="481" ht="15" hidden="0" customHeight="1">
@@ -11681,10 +11681,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C488" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D488" s="12" t="str">
-        <x:v>The text explicitly reports the same output for a given angle across all three controlled repetitions, contrasting this with variable returns during unguided movement.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E488" s="12" t="str">
         <x:v>S075_Main.pdf, physical pp. 7-8, section V; p. 8, Fig. 7c and final controlled-movement paragraph.</x:v>
@@ -11693,7 +11693,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G488" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="489" ht="24" hidden="0" customHeight="1">
@@ -11865,19 +11865,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C496" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D496" s="12" t="str">
-        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
+        <x:v>Route B—integrated assembly: the assembled nanogenerator completed 1000 cycles with peak voltage retained within 95% ± 3% of its initial value; supplementary testing extended the stability observation to about 5000 cycles.</x:v>
       </x:c>
       <x:c r="E496" s="12" t="str">
-        <x:v>PDF pp. 3–8; Figs. 1–6; cited Supplementary Figs. S1–S10</x:v>
+        <x:v>S076_Main.pdf, physical pp. 6–7, Fig. 5g; Supplementary Fig. S9</x:v>
       </x:c>
       <x:c r="F496" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G496" s="12" t="str">
-        <x:v>Rule-clarification recode</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="497" ht="24" hidden="0" customHeight="1">
@@ -12049,19 +12049,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C504" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D504" s="12" t="str">
-        <x:v>Section 3.4 explicitly describes consistent response during cyclic pronunciation and subsequent tests, and constant patterns across two extensive chewing cycles.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E504" s="12" t="str">
         <x:v>S077_Main.pdf, physical p. 4, section 2.4 attachment; pp. 11-12, section 3.4/Fig. 6, especially chewing comparison.</x:v>
       </x:c>
       <x:c r="F504" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G504" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="505" ht="15" hidden="0" customHeight="1">
@@ -12233,19 +12233,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C512" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D512" s="12" t="str">
-        <x:v>Section 2.3 explicitly compares peak values and sizes and describes them as relatively uniform across the finger repetitions.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E512" s="12" t="str">
         <x:v>S078_Main.pdf, physical p. 7, section 2.3/Fig. 6a-b; S078_Supplement_01.docx.</x:v>
       </x:c>
       <x:c r="F512" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G512" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="513" ht="24" hidden="0" customHeight="1">
@@ -12420,16 +12420,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D520" s="12" t="str">
-        <x:v>The main text reports about 70% ± 5% resistance change at baseline and minimal change in response to the same bending motions after conditioning.</x:v>
+        <x:v>Route B—integrated assembly: the sensor retained approximately 70% ± 5% resistance change during the same bending motion after high-temperature, low-temperature and water-conditioning procedures, with minimal response change.</x:v>
       </x:c>
       <x:c r="E520" s="12" t="str">
-        <x:v>S079_Main.pdf, physical p. 10, Fig. 7b; p. 11, section 3.4, paragraph referring to Fig. S15.</x:v>
+        <x:v>S079_Main.pdf, physical pp. 10–11, Fig. 7b and discussion of Supplementary Fig. S15</x:v>
       </x:c>
       <x:c r="F520" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G520" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="521" ht="24" hidden="0" customHeight="1">
@@ -12610,10 +12610,10 @@
         <x:v>PDF pp. 2, 4–12; Figs. 1–8</x:v>
       </x:c>
       <x:c r="F528" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G528" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="529" ht="24" hidden="0" customHeight="1">
@@ -12797,7 +12797,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G536" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="537" ht="15" hidden="0" customHeight="1">
@@ -12978,10 +12978,10 @@
         <x:v>PDF pp. 4–12; Figs. 1–7; Supplementary Figs. S1–S5 cited</x:v>
       </x:c>
       <x:c r="F544" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G544" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="545" ht="24" hidden="0" customHeight="1">
@@ -13162,10 +13162,10 @@
         <x:v>PDF pp. 4–11; Figs. 1–8; Supplementary Figs. S1–S5 cited</x:v>
       </x:c>
       <x:c r="F552" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G552" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="553" ht="24" hidden="0" customHeight="1">
@@ -13337,19 +13337,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C560" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D560" s="12" t="str">
-        <x:v>The sensor remains intact against its film substrate after laboratory cycling. Fig. 18 sketches a lumbar use case without a corresponding repeated-wear retention dataset.</x:v>
+        <x:v>Route A—direct interface: after 3000 tensile cycles, the printed CBP/TPU sensing structure remained intact and fitted to the TPU-film substrate while the response maxima remained approximately steady.</x:v>
       </x:c>
       <x:c r="E560" s="12" t="str">
-        <x:v>S085_Main.pdf, physical pp. 3-4, setup/Fig. 4; pp. 9-10, Fig. 15; p. 12, Fig. 18/application discussion.</x:v>
+        <x:v>S085_Main.pdf, physical pp. 9–10, Figs. 15–16</x:v>
       </x:c>
       <x:c r="F560" s="12" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G560" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="561" ht="24" hidden="0" customHeight="1">
@@ -13530,10 +13530,10 @@
         <x:v>PDF pp. 2–9; Figs. 1–6; Supporting Figs. S1–S3 and Table S1 cited</x:v>
       </x:c>
       <x:c r="F568" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G568" s="12" t="str">
-        <x:v>Rule-clarification recode</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="569" ht="24" hidden="0" customHeight="1">
@@ -13705,19 +13705,19 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C576" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D576" s="12" t="str">
-        <x:v>No qualifying interface-integrity test or repeated final monolithic wearable-assembly test with a retention/failure endpoint was located.</x:v>
+        <x:v>Route A—direct interface: standardized tape peel testing measured peel force and graphene transfer, demonstrating stronger graphene–SEBS adhesion for the surface-filled structure than for the surface-coated comparator.</x:v>
       </x:c>
       <x:c r="E576" s="12" t="str">
-        <x:v>PDF pp. 2–7; Figs. 1–5; Supplementary Figs. S1–S7 cited</x:v>
+        <x:v>S087_Main.pdf, physical pp. 3–4, Fig. 1 and Supplementary Figs. S3–S4</x:v>
       </x:c>
       <x:c r="F576" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G576" s="12" t="str">
-        <x:v>Rule-clarification recode</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="577" ht="24" hidden="0" customHeight="1">
@@ -13889,10 +13889,10 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="C584" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D584" s="12" t="str">
-        <x:v>An additional cyclic test explicitly examines measurement performance; six bends show relatively stable wavelength changes. Repeated calibration tests are also reported.</x:v>
+        <x:v>Does not qualify after the complete L7 audit: the report shows qualitative waveform repetition or a wearable demonstration, but no Route A direct-interface endpoint and no Route B defined retention or failure endpoint for the final assembly.</x:v>
       </x:c>
       <x:c r="E584" s="12" t="str">
         <x:v>S088_Main.pdf, physical p. 7, cyclic-elbow paragraph; p. 10, Fig. 8 (the paragraph mislabels its figure reference as Fig. 7).</x:v>
@@ -13901,7 +13901,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="G584" s="12" t="str">
-        <x:v>Final L7 reassessment</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="585" ht="15" hidden="0" customHeight="1">
@@ -14082,10 +14082,10 @@
         <x:v>PDF pp. 10–35 of available accepted manuscript; Figs. 1–10; Tables 1–2; Supplementary Tables S1–S2 cited</x:v>
       </x:c>
       <x:c r="F592" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G592" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="593" ht="36" hidden="0" customHeight="1">
@@ -14266,10 +14266,10 @@
         <x:v>PDF pp. 2–7; Figs. 1, 3–4; Tables 1–2</x:v>
       </x:c>
       <x:c r="F600" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G600" s="12" t="str">
-        <x:v>Batch 09</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="601" ht="24" hidden="0" customHeight="1">
@@ -14450,10 +14450,10 @@
         <x:v>PDF pp. 1–8; Figs. 2, 6–11; Table 1; ESI Table S1 and Fig. S5 cited</x:v>
       </x:c>
       <x:c r="F608" s="12" t="str">
-        <x:v>Clear</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="G608" s="12" t="str">
-        <x:v>Adjudicated to Reviewer 2</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="609" ht="24" hidden="0" customHeight="1">
@@ -27151,16 +27151,16 @@
         <x:v>Skin temperature is monitored under the attached optical probe; temperature is not a deliberately varied environmental stress.</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>Code L7=1 as a quantified interface-safety endpoint and L6=0.</x:v>
+        <x:v>Superseded by the complete L7 audit. Skin-temperature monitoring is not an interface-integrity or integrated-assembly retention endpoint; final L7=0 and L6=0.</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>Moderate</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
         <x:v>PDF pp. 3–4, 9; Figs. 1, 7c, 8c</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" hidden="0" customHeight="1">
@@ -27177,7 +27177,7 @@
         <x:v>The named supplementary source was obtained and reviewed.</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>Final decision: 1; Peel-off force was measured in newtons over time for coated, embedded and unmodified TPE sensing units attached to test tape.</x:v>
+        <x:v>Final L7=1 through Route A. The supplementary peel-force experiment directly evaluates the integral CNT–TPE sensing interface.</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>Resolved</x:v>
@@ -27186,7 +27186,7 @@
         <x:v>Supplementary Fig. S2, SI p. 2</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
-        <x:v>Supplement verified 2026-09-03</x:v>
+        <x:v>Complete two-route L7 audit</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
@@ -29106,16 +29106,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J2" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K2" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L2" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M2" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N2" s="13" t="n">
         <x:v>0</x:v>
@@ -29194,16 +29194,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K4" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="14" t="n">
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M4" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N4" s="13" t="n">
         <x:v>0</x:v>
@@ -29854,16 +29854,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K19" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L19" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N19" s="13" t="n">
         <x:v>0</x:v>
@@ -30206,16 +30206,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J27" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K27" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L27" s="14" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N27" s="13" t="n">
         <x:v>0</x:v>
@@ -30250,16 +30250,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J28" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K28" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L28" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="N28" s="13" t="n">
         <x:v>0</x:v>
@@ -30426,16 +30426,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J32" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K32" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L32" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M32" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N32" s="13" t="n">
         <x:v>0</x:v>
@@ -30470,16 +30470,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K33" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L33" s="14" t="n">
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M33" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N33" s="13" t="n">
         <x:v>0</x:v>
@@ -30602,16 +30602,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J36" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K36" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L36" s="14" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.375</x:v>
       </x:c>
       <x:c r="M36" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N36" s="13" t="n">
         <x:v>0</x:v>
@@ -30690,16 +30690,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J38" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K38" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L38" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M38" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N38" s="13" t="n">
         <x:v>0</x:v>
@@ -30822,16 +30822,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J41" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K41" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L41" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M41" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N41" s="13" t="n">
         <x:v>0</x:v>
@@ -30954,16 +30954,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J44" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K44" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L44" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M44" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N44" s="13" t="n">
         <x:v>0</x:v>
@@ -30998,16 +30998,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J45" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K45" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L45" s="14" t="n">
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M45" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N45" s="13" t="n">
         <x:v>0</x:v>
@@ -31042,16 +31042,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J46" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K46" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L46" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M46" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N46" s="13" t="n">
         <x:v>0</x:v>
@@ -31130,16 +31130,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J48" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K48" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L48" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M48" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N48" s="13" t="n">
         <x:v>0</x:v>
@@ -31306,16 +31306,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J52" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K52" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L52" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M52" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N52" s="13" t="n">
         <x:v>0</x:v>
@@ -31438,16 +31438,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J55" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K55" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L55" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M55" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N55" s="13" t="n">
         <x:v>0</x:v>
@@ -31482,16 +31482,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J56" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K56" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L56" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M56" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N56" s="13" t="n">
         <x:v>0</x:v>
@@ -31526,16 +31526,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J57" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K57" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L57" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="M57" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N57" s="13" t="n">
         <x:v>0</x:v>
@@ -31570,16 +31570,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J58" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K58" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L58" s="14" t="n">
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M58" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N58" s="13" t="n">
         <x:v>0</x:v>
@@ -31658,16 +31658,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J60" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K60" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L60" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M60" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N60" s="13" t="n">
         <x:v>0</x:v>
@@ -31746,16 +31746,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J62" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K62" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L62" s="14" t="n">
-        <x:v>0.875</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M62" s="13" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N62" s="13" t="n">
         <x:v>0</x:v>
@@ -31790,16 +31790,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J63" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K63" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L63" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M63" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N63" s="13" t="n">
         <x:v>0</x:v>
@@ -31834,16 +31834,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J64" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K64" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L64" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M64" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N64" s="13" t="n">
         <x:v>0</x:v>
@@ -31878,16 +31878,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J65" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K65" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L65" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M65" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N65" s="13" t="n">
         <x:v>0</x:v>
@@ -32142,16 +32142,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J71" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K71" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L71" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="M71" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N71" s="13" t="n">
         <x:v>0</x:v>
@@ -32230,16 +32230,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J73" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K73" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L73" s="14" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M73" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N73" s="13" t="n">
         <x:v>0</x:v>
@@ -32274,16 +32274,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J74" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K74" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L74" s="14" t="n">
-        <x:v>0.625</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M74" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N74" s="13" t="n">
         <x:v>0</x:v>
@@ -35264,15 +35264,12 @@
         <x:v>L1</x:v>
       </x:c>
       <x:c r="B2" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!D2:D77,1)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="C2" s="17" t="n">
-        <x:f>B2/76</x:f>
         <x:v>0.4342105263157895</x:v>
       </x:c>
       <x:c r="D2" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!D2:D77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="12" t="str">
@@ -35293,15 +35290,12 @@
         <x:v>L2</x:v>
       </x:c>
       <x:c r="B3" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!E2:E77,1)</x:f>
         <x:v>75</x:v>
       </x:c>
       <x:c r="C3" s="17" t="n">
-        <x:f>B3/76</x:f>
         <x:v>0.9868421052631579</x:v>
       </x:c>
       <x:c r="D3" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!E2:E77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
@@ -35322,15 +35316,12 @@
         <x:v>L3</x:v>
       </x:c>
       <x:c r="B4" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!F2:F77,1)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="C4" s="17" t="n">
-        <x:f>B4/76</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!F2:F77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
@@ -35351,15 +35342,12 @@
         <x:v>L4</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!G2:G77,1)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="C5" s="17" t="n">
-        <x:f>B5/76</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!G2:G77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
@@ -35380,15 +35368,12 @@
         <x:v>L5</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!H2:H77,1)</x:f>
         <x:v>62</x:v>
       </x:c>
       <x:c r="C6" s="17" t="n">
-        <x:f>B6/76</x:f>
         <x:v>0.8157894736842105</x:v>
       </x:c>
       <x:c r="D6" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!H2:H77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
@@ -35409,15 +35394,12 @@
         <x:v>L6</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!I2:I77,1)</x:f>
         <x:v>31</x:v>
       </x:c>
       <x:c r="C7" s="17" t="n">
-        <x:f>B7/76</x:f>
         <x:v>0.40789473684210525</x:v>
       </x:c>
       <x:c r="D7" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!I2:I77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
@@ -35438,15 +35420,12 @@
         <x:v>L7</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!J2:J77,1)</x:f>
-        <x:v>29</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
-        <x:f>B8/76</x:f>
-        <x:v>0.3815789473684211</x:v>
+        <x:v>0.2631578947368421</x:v>
       </x:c>
       <x:c r="D8" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!J2:J77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
@@ -35467,15 +35446,12 @@
         <x:v>L8</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!K2:K77,1)</x:f>
         <x:v>17</x:v>
       </x:c>
       <x:c r="C9" s="17" t="n">
-        <x:f>B9/76</x:f>
         <x:v>0.2236842105263158</x:v>
       </x:c>
       <x:c r="D9" s="13" t="n">
-        <x:f>COUNTIF('Study REB Profile'!K2:K77,"U")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
@@ -35530,8 +35506,7 @@
         <x:v>Mean R</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>AVERAGE('Study REB Profile'!L2:L77)</x:f>
-        <x:v>0.65625</x:v>
+        <x:v>0.6414473684210527</x:v>
       </x:c>
       <x:c r="C13" s="12"/>
       <x:c r="D13" s="12"/>
@@ -35545,7 +35520,6 @@
         <x:v>Minimum R</x:v>
       </x:c>
       <x:c r="B14" s="14" t="n">
-        <x:f>MIN('Study REB Profile'!L2:L77)</x:f>
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="C14" s="12"/>
@@ -35560,7 +35534,6 @@
         <x:v>Maximum R</x:v>
       </x:c>
       <x:c r="B15" s="14" t="n">
-        <x:f>MAX('Study REB Profile'!L2:L77)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C15" s="12"/>
@@ -35575,7 +35548,6 @@
         <x:v>Studies</x:v>
       </x:c>
       <x:c r="B16" s="13" t="n">
-        <x:f>COUNTA('Study REB Profile'!B2:B77)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="C16" s="12"/>
@@ -35590,7 +35562,6 @@
         <x:v>Profiles with final R</x:v>
       </x:c>
       <x:c r="B17" s="13" t="n">
-        <x:f>COUNT('Study REB Profile'!L2:L77)</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="C17" s="12"/>
@@ -35605,7 +35576,6 @@
         <x:v>Unresolved REB items</x:v>
       </x:c>
       <x:c r="B18" s="13" t="n">
-        <x:f>SUM('Study REB Profile'!N2:N77)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="12"/>

</xml_diff>

<commit_message>
Address reviewer comments 2 through 4
</commit_message>
<xml_diff>
--- a/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
+++ b/Supplementary_Data_1_Master_Extraction_76_Studies.xlsx
@@ -2,25 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rba012b6e3f4247af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R6d34eeb97bf4481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="Rb6288531edf54367"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="R3e65555e28aa49d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="R8ee214fdfb9448d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="Ref212166c5954855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="Racdcd1782a134081"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="R010e7183140e44be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="R9b28380804bd4299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Rcb363ef7bb7341c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="Rd974bc0fbf3d4b4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="Re40a743cc35d48df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R2c403d0a5a09488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rfdef40847538455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="Rbe614843c17d4339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Re437d45c411d497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R27fbd55db8b54216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R77fc1e83dcf54c34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="Rfd43a54c4d574780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R11765d36c61c41ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study Register" sheetId="2" r:id="R67422f46fa4a4be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility" sheetId="3" r:id="R34f887ddaa704434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensor Configurations" sheetId="4" r:id="Rdc559b8dda03423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="5" r:id="Rb3004f39100d45de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Printing" sheetId="6" r:id="R9402819181874d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration" sheetId="7" r:id="Rec90e576bbdd4691"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="8" r:id="Ra07b657765a14855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantitative Outcomes" sheetId="9" r:id="Rae2ef463b8ab4f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REB Coding" sheetId="10" r:id="Rb397f3baa268453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk of Bias" sheetId="11" r:id="R32c5c64eaf04443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambiguity Log" sheetId="12" r:id="R962dd6507eac45e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplement Verification" sheetId="13" r:id="R5e6aac8e497c4d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion Log" sheetId="14" r:id="Rf59c5e126ed54927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study REB Profile" sheetId="15" r:id="R1efba7a9865c4072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Completeness" sheetId="16" r:id="Red857e85500f483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthesis Summary" sheetId="17" r:id="R010184a2aa6c42b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Findings" sheetId="18" r:id="R7633b659f1d943d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural QA" sheetId="19" r:id="R59c629fdf6b940df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L6 Evidence Subtypes" sheetId="20" r:id="R7595e31abec44f90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +37,7 @@
     <x:numFmt numFmtId="201" formatCode="0.000"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -58,8 +59,18 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,8 +87,13 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -93,11 +109,25 @@
         <x:color rgb="FFB7B7B7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -135,6 +165,42 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -439,7 +505,7 @@
         <x:v>Workbook status</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>Structural validation passed: 76 studies, 608 resolved REB decisions, 608 risk judgments and 13 exclusions.</x:v>
+        <x:v>Structural validation passed: 76 studies, 608 resolved REB decisions, 608 risk judgments and 13 exclusions. L6 uses the corrected extrinsic-exposure rule; S004 is L6=0.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" hidden="0" customHeight="1">
@@ -447,7 +513,7 @@
         <x:v>Consensus provenance</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>The final profiles use the complete two-route L7 audit recorded in Supplementary Data 4. Article-specific reasons and locators are retained in REB Coding.</x:v>
+        <x:v>The final profiles use the complete two-route L7 audit and the L6 subtype audit recorded in Supplementary Data 4. S090 and S091 are flagged as borderline primary inclusions and excluded in the strict wearable-eligibility sensitivity analysis.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -805,7 +871,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Artificial-sweat pH and interferents stated; recovery/response reported.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Artificial-sweat pH and interferents stated; recovery/response reported.</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
         <x:v>PDF pp. 8-10, Fig. 6-7</x:v>
@@ -814,7 +880,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G15" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -986,19 +1052,19 @@
         <x:v>L6</x:v>
       </x:c>
       <x:c r="C23" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>Strain-rate variation is a stated use-related condition and the response is compared.</x:v>
+        <x:v>Loading rate is a parameter of the intended tensile-strain input, not an exposure extrinsic to the measurand; no qualifying L6 condition was reported.</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>PDF pp. 2–13; Figs. 1–8</x:v>
+        <x:v>PDF pp. 10-11; Fig. 6h</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G23" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>L6 consistency audit</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -1357,7 +1423,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Electrode contact pressure is a declared mounting/use condition distinct from EEG measurand; impedance response is reported.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Electrode contact pressure is a declared mounting/use condition distinct from EEG measurand; impedance response is reported.</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
         <x:v>PDF pp. 5-6, 9-10; Fig. 5</x:v>
@@ -1366,7 +1432,7 @@
         <x:v>Uncertain</x:v>
       </x:c>
       <x:c r="G39" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -2093,7 +2159,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D71" s="12" t="str">
-        <x:v>Dry versus water-moistened contact is a declared use-related condition with response comparison.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Dry versus water-moistened contact is a declared use-related condition with response comparison.</x:v>
       </x:c>
       <x:c r="E71" s="12" t="str">
         <x:v>PDF pp. 4–14; Figs. 1–17; Tables 2–3</x:v>
@@ -2102,7 +2168,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G71" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
@@ -2277,7 +2343,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="12" t="str">
-        <x:v>Daily washing/storage over 12 days with response stability is reported.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Distilled-water washing followed by room storage between daily measurements was reported. Evidence: Daily washing/storage over 12 days with response stability is reported.</x:v>
       </x:c>
       <x:c r="E79" s="12" t="str">
         <x:v>PDF pp. 3–7; Figs. 1–6; Table 1; cited SI</x:v>
@@ -2286,7 +2352,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G79" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
@@ -2461,7 +2527,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D87" s="12" t="str">
-        <x:v>20–50 °C exposure with sensor response.</x:v>
+        <x:v>In-exposure cross-sensitivity only: 20–50 °C exposure with sensor response.</x:v>
       </x:c>
       <x:c r="E87" s="12" t="str">
         <x:v>PDF pp. 4–15; Figs. 1–10; Tables 1–2</x:v>
@@ -2470,7 +2536,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G87" s="12" t="str">
-        <x:v>Batch 01</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
@@ -2829,7 +2895,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D103" s="12" t="str">
-        <x:v>Humidity and buckling/recovery exposures with output response are reported.</x:v>
+        <x:v>Both; defined reference/recovery not reported: Post-buckling recovery output was reported, but the recovery interval and reference conditioning were not specified. Evidence: Humidity and buckling/recovery exposures with output response are reported.</x:v>
       </x:c>
       <x:c r="E103" s="12" t="str">
         <x:v>PDF pp. 4-5, Fig. 4</x:v>
@@ -2838,7 +2904,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G103" s="12" t="str">
-        <x:v>Pilot</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="15" hidden="0" customHeight="1">
@@ -3197,7 +3263,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D119" s="12" t="str">
-        <x:v>Response was measured from 20–30 °C.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Response was measured from 20–30 °C.</x:v>
       </x:c>
       <x:c r="E119" s="12" t="str">
         <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
@@ -3206,7 +3272,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G119" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="15" hidden="0" customHeight="1">
@@ -3749,7 +3815,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D143" s="12" t="str">
-        <x:v>Resistance response was measured from 23% to 85% RH; the reported normalized-resistance variation was on the order of 10^-3.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Resistance response was measured from 23% to 85% RH; the reported normalized-resistance variation was on the order of 10^-3.</x:v>
       </x:c>
       <x:c r="E143" s="12" t="str">
         <x:v>Supplementary Fig. S9</x:v>
@@ -3758,7 +3824,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G143" s="12" t="str">
-        <x:v>Supplement verified 2026-09-03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="15" hidden="0" customHeight="1">
@@ -4117,7 +4183,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D159" s="12" t="str">
-        <x:v>Sensor response was compared before exposure and after 3 and 7 days at 60 °C and 80% RH; gauge factor decreased by 5.4% and 9.1%, respectively.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: The 3- and 7-day exposure time points were defined, but no return-to-reference or recovery period was reported. Evidence: Sensor response was compared before exposure and after 3 and 7 days at 60 °C and 80% RH; gauge factor decreased by 5.4% and 9.1%, respectively.</x:v>
       </x:c>
       <x:c r="E159" s="12" t="str">
         <x:v>Main article p. 7; Supplementary Fig. S4, SI p. 4</x:v>
@@ -4126,7 +4192,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G159" s="12" t="str">
-        <x:v>Supplement verified 2026-09-03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="15" hidden="0" customHeight="1">
@@ -4301,7 +4367,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D167" s="12" t="str">
-        <x:v>Temperature and repeated skin-insertion effects are reported.</x:v>
+        <x:v>Both; defined reference/recovery not reported: Response after repeated insertion was reported, but no return-to-reference condition or recovery period was defined. Evidence: Temperature and repeated skin-insertion effects are reported.</x:v>
       </x:c>
       <x:c r="E167" s="12" t="str">
         <x:v>PDF pp. 2–10; Figs. 1–6; Table 1; cited SI</x:v>
@@ -4310,7 +4376,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G167" s="12" t="str">
-        <x:v>Batch 02</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="15" hidden="0" customHeight="1">
@@ -4669,7 +4735,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D183" s="12" t="str">
-        <x:v>Fresh and 60-day-aged specimens were compared over repeated bends, giving a time/storage exposure response.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Fresh and 60-day-aged devices were compared; no return-to-reference or recovery phase was reported. Evidence: Fresh and 60-day-aged specimens were compared over repeated bends, giving a time/storage exposure response.</x:v>
       </x:c>
       <x:c r="E183" s="12" t="str">
         <x:v>PDF pp. 4–23; Figs. 3–17; Tables 2–7</x:v>
@@ -4678,7 +4744,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G183" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="15" hidden="0" customHeight="1">
@@ -5405,7 +5471,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D215" s="12" t="str">
-        <x:v>Water/ethanol washing is a declared use-related exposure with response and structural outcomes.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Response across wash/reuse cycles was reported, but no separate drying or recovery interval was defined. Evidence: Water/ethanol washing is a declared use-related exposure with response and structural outcomes.</x:v>
       </x:c>
       <x:c r="E215" s="12" t="str">
         <x:v>PDF pp. 2–9; Figs. 1–5; cited SI</x:v>
@@ -5414,7 +5480,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G215" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="15" hidden="0" customHeight="1">
@@ -5589,7 +5655,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D223" s="12" t="str">
-        <x:v>Daily washing/ambient storage over 10 days is a declared exposure with retained response.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Daily washing followed by ambient storage before subsequent measurements was reported. Evidence: Daily washing/ambient storage over 10 days is a declared exposure with retained response.</x:v>
       </x:c>
       <x:c r="E223" s="12" t="str">
         <x:v>PDF pp. 1–5; Figs. 1–4; cited SI</x:v>
@@ -5598,7 +5664,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G223" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="15" hidden="0" customHeight="1">
@@ -5773,7 +5839,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D231" s="12" t="str">
-        <x:v>Temperature 24–40 °C and concentration 0.5×–1.25× were varied with sweat-rate deviation reported.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Temperature 24–40 °C and concentration 0.5×–1.25× were varied with sweat-rate deviation reported.</x:v>
       </x:c>
       <x:c r="E231" s="12" t="str">
         <x:v>PDF pp. 2–11; Figs. 1–6; cited SI</x:v>
@@ -5782,7 +5848,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G231" s="12" t="str">
-        <x:v>Batch 03</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="232" ht="24" hidden="0" customHeight="1">
@@ -7245,7 +7311,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D295" s="12" t="str">
-        <x:v>Water and organic-solvent immersion/ultrasonication for four hours was followed by resistance measurements.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Resistance was measured after drying and cooling at 30-minute intervals. Evidence: Water and organic-solvent immersion/ultrasonication for four hours was followed by resistance measurements.</x:v>
       </x:c>
       <x:c r="E295" s="12" t="str">
         <x:v>PDF pp. 3–9; Figs. 1, 4–9; cited SI</x:v>
@@ -7254,7 +7320,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G295" s="12" t="str">
-        <x:v>Batch 04</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="296" ht="15" hidden="0" customHeight="1">
@@ -7429,7 +7495,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D303" s="12" t="str">
-        <x:v>Sensor response was quantified from 25 to 45 °C and force compensation was evaluated.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Sensor response was quantified from 25 to 45 °C and force compensation was evaluated.</x:v>
       </x:c>
       <x:c r="E303" s="12" t="str">
         <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
@@ -7438,7 +7504,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G303" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="304" ht="15" hidden="0" customHeight="1">
@@ -7613,7 +7679,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D311" s="12" t="str">
-        <x:v>The device response was measured in rooms from 6 to 40 °C.</x:v>
+        <x:v>In-exposure cross-sensitivity only: The device response was measured in rooms from 6 to 40 °C.</x:v>
       </x:c>
       <x:c r="E311" s="12" t="str">
         <x:v>PDF pp. 2–7; Figs. 1–5</x:v>
@@ -7622,7 +7688,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G311" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="312" ht="15" hidden="0" customHeight="1">
@@ -7797,7 +7863,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D319" s="12" t="str">
-        <x:v>Ambient humidity and temperature response are explicitly reported, with detail in cited supplementary figures.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Ambient humidity and temperature response are explicitly reported, with detail in cited supplementary figures.</x:v>
       </x:c>
       <x:c r="E319" s="12" t="str">
         <x:v>PDF pp. 2–12; Figs. 1–6; cited Supplementary Table S1 and Figs. S1–S21</x:v>
@@ -7806,7 +7872,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G319" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="320" ht="24" hidden="0" customHeight="1">
@@ -8533,7 +8599,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D351" s="12" t="str">
-        <x:v>Liquids, humidity and sweat-related responses were measured.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Liquids, humidity and sweat-related responses were measured.</x:v>
       </x:c>
       <x:c r="E351" s="12" t="str">
         <x:v>PDF pp. 3–15; Figs. 1–9; Tables 1–2</x:v>
@@ -8542,7 +8608,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G351" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="352" ht="15" hidden="0" customHeight="1">
@@ -8901,7 +8967,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D367" s="12" t="str">
-        <x:v>Temperature, humidity and artificial-sweat responses were measured.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Temperature, humidity and artificial-sweat responses were measured.</x:v>
       </x:c>
       <x:c r="E367" s="12" t="str">
         <x:v>PDF pp. 3–13; Figs. 1–8; cited Supplementary Table S1</x:v>
@@ -8910,7 +8976,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G367" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="368" ht="24" hidden="0" customHeight="1">
@@ -9085,7 +9151,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D375" s="12" t="str">
-        <x:v>Electrodes were tested dry and after declared water moistening with quantitative impedance/SNR response.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Electrodes were tested dry and after declared water moistening with quantitative impedance/SNR response.</x:v>
       </x:c>
       <x:c r="E375" s="12" t="str">
         <x:v>PDF pp. 3–15; Figs. 1–9; cited Supplementary Table S1</x:v>
@@ -9094,7 +9160,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G375" s="12" t="str">
-        <x:v>Batch 05</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="376" ht="24" hidden="0" customHeight="1">
@@ -9453,7 +9519,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D391" s="12" t="str">
-        <x:v>Response was compared between stated with-wear/without-wear assembly-loading states.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Response was compared between stated with-wear/without-wear assembly-loading states.</x:v>
       </x:c>
       <x:c r="E391" s="12" t="str">
         <x:v>PDF pp. 2–11; Figs. 1–13; Table 1</x:v>
@@ -9462,7 +9528,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G391" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="392" ht="15" hidden="0" customHeight="1">
@@ -10189,7 +10255,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D423" s="12" t="str">
-        <x:v>Walking, jogging and stair use provide declared use-related activity exposure with quantified response.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Walking, jogging and stair use provide declared use-related activity exposure with quantified response.</x:v>
       </x:c>
       <x:c r="E423" s="12" t="str">
         <x:v>PDF pp. 2–8; Figs. 1–8; Table I</x:v>
@@ -10198,7 +10264,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G423" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="424" ht="15" hidden="0" customHeight="1">
@@ -10373,7 +10439,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D431" s="12" t="str">
-        <x:v>Temperature and humidity were deliberately varied and the output was reported.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Temperature and humidity were deliberately varied and the output was reported.</x:v>
       </x:c>
       <x:c r="E431" s="12" t="str">
         <x:v>PDF pp. 2–9; Figs. 1–8</x:v>
@@ -10382,7 +10448,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G431" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="432" ht="15" hidden="0" customHeight="1">
@@ -10741,7 +10807,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D447" s="12" t="str">
-        <x:v>Water/detergent washing for 30 min was followed by output measurement.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Output after 30 minutes of hand washing was reported without a stated drying or recovery interval. Evidence: Water/detergent washing for 30 min was followed by output measurement.</x:v>
       </x:c>
       <x:c r="E447" s="12" t="str">
         <x:v>PDF pp. 2–12; Figs. 1–11; Table 1; cited SI</x:v>
@@ -10750,7 +10816,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G447" s="12" t="str">
-        <x:v>Batch 06</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="448" ht="15" hidden="0" customHeight="1">
@@ -10925,7 +10991,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D455" s="12" t="str">
-        <x:v>Temperature and RH were deliberately varied with sensor response reported.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Temperature and RH were deliberately varied with sensor response reported.</x:v>
       </x:c>
       <x:c r="E455" s="12" t="str">
         <x:v>PDF pp. 3–9; Figs. 1–12; Tables I–III</x:v>
@@ -10934,7 +11000,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G455" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="456" ht="15" hidden="0" customHeight="1">
@@ -11477,7 +11543,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D479" s="12" t="str">
-        <x:v>Temperature was deliberately varied as a cross-sensitivity condition for the strain/wearable sensor.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Temperature was deliberately varied as a cross-sensitivity condition for the strain/wearable sensor.</x:v>
       </x:c>
       <x:c r="E479" s="12" t="str">
         <x:v>PDF pp. 3–9; Figs. 1–13</x:v>
@@ -11486,7 +11552,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G479" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="480" ht="15" hidden="0" customHeight="1">
@@ -11661,7 +11727,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D487" s="12" t="str">
-        <x:v>Controlled temperature and RH cycles report response for all three configurations.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Controlled temperature and RH cycles report response for all three configurations.</x:v>
       </x:c>
       <x:c r="E487" s="12" t="str">
         <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
@@ -11670,7 +11736,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G487" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="488" ht="15" hidden="0" customHeight="1">
@@ -12397,7 +12463,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D519" s="12" t="str">
-        <x:v>Performance was measured after 40 °C, −35 °C and 24-h water immersion/rubbing exposures.</x:v>
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Post-exposure response followed temperature, water-immersion and rubbing challenges without a stated return-to-reference or recovery period. Evidence: Performance was measured after 40 °C, −35 °C and 24-h water immersion/rubbing exposures.</x:v>
       </x:c>
       <x:c r="E519" s="12" t="str">
         <x:v>PDF pp. 2–12; Figs. 1–8; Supplementary Figs. S1–S15 cited</x:v>
@@ -12406,7 +12472,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G519" s="12" t="str">
-        <x:v>Batch 07</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="520" ht="24" hidden="0" customHeight="1">
@@ -14053,7 +14119,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D591" s="12" t="str">
-        <x:v>Conductivity was measured and reported across a stated 20–80 °C exposure.</x:v>
+        <x:v>In-exposure cross-sensitivity only: Conductivity was measured and reported across a stated 20–80 °C exposure.</x:v>
       </x:c>
       <x:c r="E591" s="12" t="str">
         <x:v>PDF pp. 10–35 of available accepted manuscript; Figs. 1–10; Tables 1–2; Supplementary Tables S1–S2 cited</x:v>
@@ -14062,7 +14128,7 @@
         <x:v>Clear</x:v>
       </x:c>
       <x:c r="G591" s="12" t="str">
-        <x:v>Batch 08</x:v>
+        <x:v>L6 subtype audit</x:v>
       </x:c>
     </x:row>
     <x:row r="592" ht="36" hidden="0" customHeight="1">
@@ -29191,7 +29257,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J4" s="13" t="n">
         <x:v>0</x:v>
@@ -29200,10 +29266,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="14" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="M4" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N4" s="13" t="n">
         <x:v>0</x:v>
@@ -35394,10 +35460,12 @@
         <x:v>L6</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>31</x:v>
+        <x:f>SUM('Study REB Profile'!I2:I77)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C7" s="17" t="n">
-        <x:v>0.40789473684210525</x:v>
+        <x:f>B7/76</x:f>
+        <x:v>0.39473684210526316</x:v>
       </x:c>
       <x:c r="D7" s="13" t="n">
         <x:v>0</x:v>
@@ -35506,7 +35574,8 @@
         <x:v>Mean R</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:v>0.6414473684210527</x:v>
+        <x:f>AVERAGE('Study REB Profile'!L2:L77)</x:f>
+        <x:v>0.6398026315789473</x:v>
       </x:c>
       <x:c r="C13" s="12"/>
       <x:c r="D13" s="12"/>
@@ -35584,6 +35653,126 @@
       <x:c r="F18" s="12"/>
       <x:c r="G18" s="12"/>
       <x:c r="H18" s="12"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="str">
+        <x:v>L6 evidence subtype</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>Percentage of 76 studies</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="25" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="B21" s="25" t="n">
+        <x:f>COUNTIF('L6 Evidence Subtypes'!E2:E31,A21)</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C21" s="26" t="n">
+        <x:f>B21/76</x:f>
+        <x:v>0.2631578947368421</x:v>
+      </x:c>
+      <x:c r="D21" s="25" t="str">
+        <x:v>Response measured during an extrinsic condition; no post-exposure retention endpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="25" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="B22" s="25" t="n">
+        <x:f>COUNTIF('L6 Evidence Subtypes'!E2:E31,A22)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C22" s="26" t="n">
+        <x:f>B22/76</x:f>
+        <x:v>0.10526315789473684</x:v>
+      </x:c>
+      <x:c r="D22" s="25" t="str">
+        <x:v>Response measured after the declared exposure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="25" t="str">
+        <x:v>Both</x:v>
+      </x:c>
+      <x:c r="B23" s="25" t="n">
+        <x:f>COUNTIF('L6 Evidence Subtypes'!E2:E31,A23)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C23" s="26" t="n">
+        <x:f>B23/76</x:f>
+        <x:v>0.02631578947368421</x:v>
+      </x:c>
+      <x:c r="D23" s="25" t="str">
+        <x:v>The study reported during-exposure and post-exposure evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="25" t="str">
+        <x:v>Post-exposure studies with defined reference/recovery</x:v>
+      </x:c>
+      <x:c r="B24" s="25" t="n">
+        <x:f>COUNTIF('L6 Evidence Subtypes'!H2:H31,"Yes")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="n">
+        <x:f>B24/10</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D24" s="25" t="str">
+        <x:v>Denominator is the 10 studies with any post-exposure retention evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="25" t="str">
+        <x:v>L7 Route A--direct interface</x:v>
+      </x:c>
+      <x:c r="B25" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="n">
+        <x:v>0.13157894736842105</x:v>
+      </x:c>
+      <x:c r="D25" s="25" t="str">
+        <x:v>Direct interface endpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="25" t="str">
+        <x:v>L7 Route B--integrated assembly</x:v>
+      </x:c>
+      <x:c r="B26" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="n">
+        <x:v>0.13157894736842105</x:v>
+      </x:c>
+      <x:c r="D26" s="25" t="str">
+        <x:v>Repeated final-assembly test with a retention/failure endpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="25" t="str">
+        <x:v>Borderline wearable strict-sensitivity set</x:v>
+      </x:c>
+      <x:c r="B27" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C27" s="26" t="n">
+        <x:v>0.02631578947368421</x:v>
+      </x:c>
+      <x:c r="D27" s="25" t="str">
+        <x:v>S090 and S091 are retained in the primary corpus and excluded in the stricter sensitivity analysis.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38777,6 +38966,1237 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="31" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="64" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="35" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" hidden="0" customHeight="1">
+      <x:c r="A1" s="33" t="str">
+        <x:v>Synthesis ID</x:v>
+      </x:c>
+      <x:c r="B1" s="33" t="str">
+        <x:v>Study ID</x:v>
+      </x:c>
+      <x:c r="C1" s="33" t="str">
+        <x:v>Citation</x:v>
+      </x:c>
+      <x:c r="D1" s="33" t="str">
+        <x:v>L6 decision</x:v>
+      </x:c>
+      <x:c r="E1" s="33" t="str">
+        <x:v>Evidence subtype</x:v>
+      </x:c>
+      <x:c r="F1" s="33" t="str">
+        <x:v>In-exposure cross-sensitivity</x:v>
+      </x:c>
+      <x:c r="G1" s="33" t="str">
+        <x:v>Post-exposure retention</x:v>
+      </x:c>
+      <x:c r="H1" s="33" t="str">
+        <x:v>Defined reference/recovery reported</x:v>
+      </x:c>
+      <x:c r="I1" s="33" t="str">
+        <x:v>Reference/recovery detail</x:v>
+      </x:c>
+      <x:c r="J1" s="33" t="str">
+        <x:v>Evidence basis</x:v>
+      </x:c>
+      <x:c r="K1" s="33" t="str">
+        <x:v>Locator</x:v>
+      </x:c>
+      <x:c r="L1" s="30"/>
+      <x:c r="M1" s="32" t="str">
+        <x:v>Audit summary</x:v>
+      </x:c>
+      <x:c r="N1" s="32" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" hidden="0" customHeight="1">
+      <x:c r="A2" s="30" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B2" s="30" t="str">
+        <x:v>S002</x:v>
+      </x:c>
+      <x:c r="C2" s="30" t="str">
+        <x:v>Koukouviti et al. (2022)</x:v>
+      </x:c>
+      <x:c r="D2" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F2" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G2" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H2" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I2" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J2" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Artificial-sweat pH and interferents stated; recovery/response reported.</x:v>
+      </x:c>
+      <x:c r="K2" s="30" t="str">
+        <x:v>PDF pp. 8-10, Fig. 6-7</x:v>
+      </x:c>
+      <x:c r="L2" s="30"/>
+      <x:c r="M2" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="N2" s="30" t="n">
+        <x:f>COUNTIF(E2:E31,M2)</x:f>
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" hidden="0" customHeight="1">
+      <x:c r="A3" s="30" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="30" t="str">
+        <x:v>S007</x:v>
+      </x:c>
+      <x:c r="C3" s="30" t="str">
+        <x:v>Velcescu et al. (2019)</x:v>
+      </x:c>
+      <x:c r="D3" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F3" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G3" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H3" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I3" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J3" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Electrode contact pressure is a declared mounting/use condition distinct from EEG measurand; impedance response is reported.</x:v>
+      </x:c>
+      <x:c r="K3" s="30" t="str">
+        <x:v>PDF pp. 5-6, 9-10; Fig. 5</x:v>
+      </x:c>
+      <x:c r="L3" s="30"/>
+      <x:c r="M3" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="N3" s="30" t="n">
+        <x:f>COUNTIF(E2:E31,M3)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" hidden="0" customHeight="1">
+      <x:c r="A4" s="30" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B4" s="30" t="str">
+        <x:v>S012</x:v>
+      </x:c>
+      <x:c r="C4" s="30" t="str">
+        <x:v>Wolterink et al. (2020)</x:v>
+      </x:c>
+      <x:c r="D4" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F4" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G4" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H4" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I4" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J4" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Dry versus water-moistened contact is a declared use-related condition with response comparison.</x:v>
+      </x:c>
+      <x:c r="K4" s="30" t="str">
+        <x:v>PDF pp. 4–14; Figs. 1–17; Tables 2–3</x:v>
+      </x:c>
+      <x:c r="L4" s="30"/>
+      <x:c r="M4" s="30" t="str">
+        <x:v>Both</x:v>
+      </x:c>
+      <x:c r="N4" s="30" t="n">
+        <x:f>COUNTIF(E2:E31,M4)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="36" hidden="0" customHeight="1">
+      <x:c r="A5" s="30" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B5" s="30" t="str">
+        <x:v>S013</x:v>
+      </x:c>
+      <x:c r="C5" s="30" t="str">
+        <x:v>Poulladofonou et al. (2022)</x:v>
+      </x:c>
+      <x:c r="D5" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F5" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G5" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H5" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I5" s="30" t="str">
+        <x:v>Distilled-water washing followed by room storage between daily measurements was reported.</x:v>
+      </x:c>
+      <x:c r="J5" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Distilled-water washing followed by room storage between daily measurements was reported. Evidence: Daily washing/storage over 12 days with response stability is reported.</x:v>
+      </x:c>
+      <x:c r="K5" s="30" t="str">
+        <x:v>PDF pp. 3–7; Figs. 1–6; Table 1; cited SI</x:v>
+      </x:c>
+      <x:c r="L5" s="30"/>
+      <x:c r="M5" s="30" t="str">
+        <x:v>Any post-exposure retention</x:v>
+      </x:c>
+      <x:c r="N5" s="30" t="n">
+        <x:f>COUNTIF(G2:G31,"Yes")</x:f>
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="30" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>S014</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>Dimo et al. (2025)</x:v>
+      </x:c>
+      <x:c r="D6" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F6" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G6" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H6" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I6" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J6" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: 20–50 °C exposure with sensor response.</x:v>
+      </x:c>
+      <x:c r="K6" s="30" t="str">
+        <x:v>PDF pp. 4–15; Figs. 1–10; Tables 1–2</x:v>
+      </x:c>
+      <x:c r="L6" s="30"/>
+      <x:c r="M6" s="30" t="str">
+        <x:v>Defined reference/recovery reported</x:v>
+      </x:c>
+      <x:c r="N6" s="30" t="n">
+        <x:f>COUNTIF(H2:H31,"Yes")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="36" hidden="0" customHeight="1">
+      <x:c r="A7" s="30" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>S017</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>Zhang and Ma (2025)</x:v>
+      </x:c>
+      <x:c r="D7" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="30" t="str">
+        <x:v>Both</x:v>
+      </x:c>
+      <x:c r="F7" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G7" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H7" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I7" s="30" t="str">
+        <x:v>Post-buckling recovery output was reported, but the recovery interval and reference conditioning were not specified.</x:v>
+      </x:c>
+      <x:c r="J7" s="30" t="str">
+        <x:v>Both; defined reference/recovery not reported: Post-buckling recovery output was reported, but the recovery interval and reference conditioning were not specified. Evidence: Humidity and buckling/recovery exposures with output response are reported.</x:v>
+      </x:c>
+      <x:c r="K7" s="30" t="str">
+        <x:v>PDF pp. 4-5, Fig. 4</x:v>
+      </x:c>
+      <x:c r="L7" s="30"/>
+      <x:c r="M7" s="30"/>
+      <x:c r="N7" s="30"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="30" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>S019</x:v>
+      </x:c>
+      <x:c r="C8" s="30" t="str">
+        <x:v>Vu et al. (2021)</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F8" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G8" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H8" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I8" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J8" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Response was measured from 20–30 °C.</x:v>
+      </x:c>
+      <x:c r="K8" s="30" t="str">
+        <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
+      </x:c>
+      <x:c r="L8" s="30"/>
+      <x:c r="M8" s="30"/>
+      <x:c r="N8" s="30"/>
+    </x:row>
+    <x:row r="9" ht="24" hidden="0" customHeight="1">
+      <x:c r="A9" s="30" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>S022</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>Yan et al. (2025)</x:v>
+      </x:c>
+      <x:c r="D9" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F9" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G9" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H9" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I9" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J9" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Resistance response was measured from 23% to 85% RH; the reported normalized-resistance variation was on the order of 10^-3.</x:v>
+      </x:c>
+      <x:c r="K9" s="30" t="str">
+        <x:v>Supplementary Fig. S9</x:v>
+      </x:c>
+      <x:c r="L9" s="30"/>
+      <x:c r="M9" s="30"/>
+      <x:c r="N9" s="30"/>
+    </x:row>
+    <x:row r="10" ht="48" hidden="0" customHeight="1">
+      <x:c r="A10" s="30" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>S024</x:v>
+      </x:c>
+      <x:c r="C10" s="30" t="str">
+        <x:v>Han et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F10" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G10" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H10" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I10" s="30" t="str">
+        <x:v>The 3- and 7-day exposure time points were defined, but no return-to-reference or recovery period was reported.</x:v>
+      </x:c>
+      <x:c r="J10" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: The 3- and 7-day exposure time points were defined, but no return-to-reference or recovery period was reported. Evidence: Sensor response was compared before exposure and after 3 and 7 days at 60 °C and 80% RH; gauge factor decreased by 5.4% and 9.1%, respectively.</x:v>
+      </x:c>
+      <x:c r="K10" s="30" t="str">
+        <x:v>Main article p. 7; Supplementary Fig. S4, SI p. 4</x:v>
+      </x:c>
+      <x:c r="L10" s="30"/>
+      <x:c r="M10" s="30"/>
+      <x:c r="N10" s="30"/>
+    </x:row>
+    <x:row r="11" ht="36" hidden="0" customHeight="1">
+      <x:c r="A11" s="30" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>S025</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>Wei et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D11" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="30" t="str">
+        <x:v>Both</x:v>
+      </x:c>
+      <x:c r="F11" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G11" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H11" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I11" s="30" t="str">
+        <x:v>Response after repeated insertion was reported, but no return-to-reference condition or recovery period was defined.</x:v>
+      </x:c>
+      <x:c r="J11" s="30" t="str">
+        <x:v>Both; defined reference/recovery not reported: Response after repeated insertion was reported, but no return-to-reference condition or recovery period was defined. Evidence: Temperature and repeated skin-insertion effects are reported.</x:v>
+      </x:c>
+      <x:c r="K11" s="30" t="str">
+        <x:v>PDF pp. 2–10; Figs. 1–6; Table 1; cited SI</x:v>
+      </x:c>
+      <x:c r="L11" s="30"/>
+      <x:c r="M11" s="30"/>
+      <x:c r="N11" s="30"/>
+    </x:row>
+    <x:row r="12" ht="48" hidden="0" customHeight="1">
+      <x:c r="A12" s="30" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="str">
+        <x:v>S029</x:v>
+      </x:c>
+      <x:c r="C12" s="30" t="str">
+        <x:v>Özkurt et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D12" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F12" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H12" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I12" s="30" t="str">
+        <x:v>Fresh and 60-day-aged devices were compared; no return-to-reference or recovery phase was reported.</x:v>
+      </x:c>
+      <x:c r="J12" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Fresh and 60-day-aged devices were compared; no return-to-reference or recovery phase was reported. Evidence: Fresh and 60-day-aged specimens were compared over repeated bends, giving a time/storage exposure response.</x:v>
+      </x:c>
+      <x:c r="K12" s="30" t="str">
+        <x:v>PDF pp. 4–23; Figs. 3–17; Tables 2–7</x:v>
+      </x:c>
+      <x:c r="L12" s="30"/>
+      <x:c r="M12" s="30"/>
+      <x:c r="N12" s="30"/>
+    </x:row>
+    <x:row r="13" ht="48" hidden="0" customHeight="1">
+      <x:c r="A13" s="30" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>S034</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>Zhang et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D13" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H13" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I13" s="30" t="str">
+        <x:v>Response across wash/reuse cycles was reported, but no separate drying or recovery interval was defined.</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Response across wash/reuse cycles was reported, but no separate drying or recovery interval was defined. Evidence: Water/ethanol washing is a declared use-related exposure with response and structural outcomes.</x:v>
+      </x:c>
+      <x:c r="K13" s="30" t="str">
+        <x:v>PDF pp. 2–9; Figs. 1–5; cited SI</x:v>
+      </x:c>
+      <x:c r="L13" s="30"/>
+      <x:c r="M13" s="30"/>
+      <x:c r="N13" s="30"/>
+    </x:row>
+    <x:row r="14" ht="36" hidden="0" customHeight="1">
+      <x:c r="A14" s="30" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>S035</x:v>
+      </x:c>
+      <x:c r="C14" s="30" t="str">
+        <x:v>Katseli et al. (2021)</x:v>
+      </x:c>
+      <x:c r="D14" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F14" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G14" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H14" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I14" s="30" t="str">
+        <x:v>Daily washing followed by ambient storage before subsequent measurements was reported.</x:v>
+      </x:c>
+      <x:c r="J14" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Daily washing followed by ambient storage before subsequent measurements was reported. Evidence: Daily washing/ambient storage over 10 days is a declared exposure with retained response.</x:v>
+      </x:c>
+      <x:c r="K14" s="30" t="str">
+        <x:v>PDF pp. 1–5; Figs. 1–4; cited SI</x:v>
+      </x:c>
+      <x:c r="L14" s="30"/>
+      <x:c r="M14" s="30"/>
+      <x:c r="N14" s="30"/>
+    </x:row>
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
+      <x:c r="A15" s="30" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>S036</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>Xuan et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F15" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G15" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I15" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J15" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Temperature 24–40 °C and concentration 0.5×–1.25× were varied with sweat-rate deviation reported.</x:v>
+      </x:c>
+      <x:c r="K15" s="30" t="str">
+        <x:v>PDF pp. 2–11; Figs. 1–6; cited SI</x:v>
+      </x:c>
+      <x:c r="L15" s="30"/>
+      <x:c r="M15" s="30"/>
+      <x:c r="N15" s="30"/>
+    </x:row>
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
+      <x:c r="A16" s="30" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>S048</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>Gunasekaran et al. (2022)</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F16" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G16" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H16" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I16" s="30" t="str">
+        <x:v>Resistance was measured after drying and cooling at 30-minute intervals.</x:v>
+      </x:c>
+      <x:c r="J16" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery reported: Resistance was measured after drying and cooling at 30-minute intervals. Evidence: Water and organic-solvent immersion/ultrasonication for four hours was followed by resistance measurements.</x:v>
+      </x:c>
+      <x:c r="K16" s="30" t="str">
+        <x:v>PDF pp. 3–9; Figs. 1, 4–9; cited SI</x:v>
+      </x:c>
+      <x:c r="L16" s="30"/>
+      <x:c r="M16" s="30"/>
+      <x:c r="N16" s="30"/>
+    </x:row>
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
+      <x:c r="A17" s="30" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>S050</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>Leal-Junior et al. (2018)</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F17" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G17" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H17" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I17" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J17" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Sensor response was quantified from 25 to 45 °C and force compensation was evaluated.</x:v>
+      </x:c>
+      <x:c r="K17" s="30" t="str">
+        <x:v>PDF pp. 3–10; Figs. 1–8</x:v>
+      </x:c>
+      <x:c r="L17" s="30"/>
+      <x:c r="M17" s="30"/>
+      <x:c r="N17" s="30"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="30" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="str">
+        <x:v>S051</x:v>
+      </x:c>
+      <x:c r="C18" s="30" t="str">
+        <x:v>Ota et al. (2017)</x:v>
+      </x:c>
+      <x:c r="D18" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F18" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G18" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H18" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I18" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J18" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: The device response was measured in rooms from 6 to 40 °C.</x:v>
+      </x:c>
+      <x:c r="K18" s="30" t="str">
+        <x:v>PDF pp. 2–7; Figs. 1–5</x:v>
+      </x:c>
+      <x:c r="L18" s="30"/>
+      <x:c r="M18" s="30"/>
+      <x:c r="N18" s="30"/>
+    </x:row>
+    <x:row r="19" ht="36" hidden="0" customHeight="1">
+      <x:c r="A19" s="30" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>S052</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>Li et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D19" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F19" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G19" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H19" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I19" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J19" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Ambient humidity and temperature response are explicitly reported, with detail in cited supplementary figures.</x:v>
+      </x:c>
+      <x:c r="K19" s="30" t="str">
+        <x:v>PDF pp. 2–12; Figs. 1–6; cited Supplementary Table S1 and Figs. S1–S21</x:v>
+      </x:c>
+      <x:c r="L19" s="30"/>
+      <x:c r="M19" s="30"/>
+      <x:c r="N19" s="30"/>
+    </x:row>
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="30" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>S056</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>Wei et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F20" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G20" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H20" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I20" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J20" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Liquids, humidity and sweat-related responses were measured.</x:v>
+      </x:c>
+      <x:c r="K20" s="30" t="str">
+        <x:v>PDF pp. 3–15; Figs. 1–9; Tables 1–2</x:v>
+      </x:c>
+      <x:c r="L20" s="30"/>
+      <x:c r="M20" s="30"/>
+      <x:c r="N20" s="30"/>
+    </x:row>
+    <x:row r="21" ht="24" hidden="0" customHeight="1">
+      <x:c r="A21" s="30" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>S058</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Yang et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F21" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G21" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H21" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I21" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J21" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Temperature, humidity and artificial-sweat responses were measured.</x:v>
+      </x:c>
+      <x:c r="K21" s="30" t="str">
+        <x:v>PDF pp. 3–13; Figs. 1–8; cited Supplementary Table S1</x:v>
+      </x:c>
+      <x:c r="L21" s="30"/>
+      <x:c r="M21" s="30"/>
+      <x:c r="N21" s="30"/>
+    </x:row>
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
+      <x:c r="A22" s="30" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>S059</x:v>
+      </x:c>
+      <x:c r="C22" s="30" t="str">
+        <x:v>Saroli et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D22" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F22" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G22" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H22" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I22" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J22" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Electrodes were tested dry and after declared water moistening with quantitative impedance/SNR response.</x:v>
+      </x:c>
+      <x:c r="K22" s="30" t="str">
+        <x:v>PDF pp. 3–15; Figs. 1–9; cited Supplementary Table S1</x:v>
+      </x:c>
+      <x:c r="L22" s="30"/>
+      <x:c r="M22" s="30"/>
+      <x:c r="N22" s="30"/>
+    </x:row>
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
+      <x:c r="A23" s="30" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>S061</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>Kumar et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F23" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G23" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H23" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I23" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J23" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Response was compared between stated with-wear/without-wear assembly-loading states.</x:v>
+      </x:c>
+      <x:c r="K23" s="30" t="str">
+        <x:v>PDF pp. 2–11; Figs. 1–13; Table 1</x:v>
+      </x:c>
+      <x:c r="L23" s="30"/>
+      <x:c r="M23" s="30"/>
+      <x:c r="N23" s="30"/>
+    </x:row>
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
+      <x:c r="A24" s="30" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="str">
+        <x:v>S066</x:v>
+      </x:c>
+      <x:c r="C24" s="30" t="str">
+        <x:v>Saroli et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D24" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F24" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G24" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H24" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I24" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J24" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Walking, jogging and stair use provide declared use-related activity exposure with quantified response.</x:v>
+      </x:c>
+      <x:c r="K24" s="30" t="str">
+        <x:v>PDF pp. 2–8; Figs. 1–8; Table I</x:v>
+      </x:c>
+      <x:c r="L24" s="30"/>
+      <x:c r="M24" s="30"/>
+      <x:c r="N24" s="30"/>
+    </x:row>
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
+      <x:c r="A25" s="30" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>S067</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>Yang et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D25" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F25" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G25" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H25" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I25" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J25" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Temperature and humidity were deliberately varied and the output was reported.</x:v>
+      </x:c>
+      <x:c r="K25" s="30" t="str">
+        <x:v>PDF pp. 2–9; Figs. 1–8</x:v>
+      </x:c>
+      <x:c r="L25" s="30"/>
+      <x:c r="M25" s="30"/>
+      <x:c r="N25" s="30"/>
+    </x:row>
+    <x:row r="26" ht="36" hidden="0" customHeight="1">
+      <x:c r="A26" s="30" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="str">
+        <x:v>S069</x:v>
+      </x:c>
+      <x:c r="C26" s="30" t="str">
+        <x:v>Babu et al. (2025)</x:v>
+      </x:c>
+      <x:c r="D26" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F26" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G26" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H26" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I26" s="30" t="str">
+        <x:v>Output after 30 minutes of hand washing was reported without a stated drying or recovery interval.</x:v>
+      </x:c>
+      <x:c r="J26" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Output after 30 minutes of hand washing was reported without a stated drying or recovery interval. Evidence: Water/detergent washing for 30 min was followed by output measurement.</x:v>
+      </x:c>
+      <x:c r="K26" s="30" t="str">
+        <x:v>PDF pp. 2–12; Figs. 1–11; Table 1; cited SI</x:v>
+      </x:c>
+      <x:c r="L26" s="30"/>
+      <x:c r="M26" s="30"/>
+      <x:c r="N26" s="30"/>
+    </x:row>
+    <x:row r="27" ht="24" hidden="0" customHeight="1">
+      <x:c r="A27" s="30" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>S070</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>Dimo et al. (2026)</x:v>
+      </x:c>
+      <x:c r="D27" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E27" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F27" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G27" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H27" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I27" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J27" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Temperature and RH were deliberately varied with sensor response reported.</x:v>
+      </x:c>
+      <x:c r="K27" s="30" t="str">
+        <x:v>PDF pp. 3–9; Figs. 1–12; Tables I–III</x:v>
+      </x:c>
+      <x:c r="L27" s="30"/>
+      <x:c r="M27" s="30"/>
+      <x:c r="N27" s="30"/>
+    </x:row>
+    <x:row r="28" ht="24" hidden="0" customHeight="1">
+      <x:c r="A28" s="30" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B28" s="30" t="str">
+        <x:v>S074</x:v>
+      </x:c>
+      <x:c r="C28" s="30" t="str">
+        <x:v>Lavorgna et al. (2025)</x:v>
+      </x:c>
+      <x:c r="D28" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F28" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G28" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H28" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I28" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J28" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Temperature was deliberately varied as a cross-sensitivity condition for the strain/wearable sensor.</x:v>
+      </x:c>
+      <x:c r="K28" s="30" t="str">
+        <x:v>PDF pp. 3–9; Figs. 1–13</x:v>
+      </x:c>
+      <x:c r="L28" s="30"/>
+      <x:c r="M28" s="30"/>
+      <x:c r="N28" s="30"/>
+    </x:row>
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
+      <x:c r="A29" s="30" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B29" s="30" t="str">
+        <x:v>S075</x:v>
+      </x:c>
+      <x:c r="C29" s="30" t="str">
+        <x:v>Saroli et al. (2025)</x:v>
+      </x:c>
+      <x:c r="D29" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E29" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F29" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G29" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H29" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I29" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J29" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Controlled temperature and RH cycles report response for all three configurations.</x:v>
+      </x:c>
+      <x:c r="K29" s="30" t="str">
+        <x:v>PDF pp. 2–8; Figs. 1–7</x:v>
+      </x:c>
+      <x:c r="L29" s="30"/>
+      <x:c r="M29" s="30"/>
+      <x:c r="N29" s="30"/>
+    </x:row>
+    <x:row r="30" ht="48" hidden="0" customHeight="1">
+      <x:c r="A30" s="30" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B30" s="30" t="str">
+        <x:v>S079</x:v>
+      </x:c>
+      <x:c r="C30" s="30" t="str">
+        <x:v>Han et al. (2024)</x:v>
+      </x:c>
+      <x:c r="D30" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="30" t="str">
+        <x:v>Post-exposure retention only</x:v>
+      </x:c>
+      <x:c r="F30" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G30" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H30" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I30" s="30" t="str">
+        <x:v>Post-exposure response followed temperature, water-immersion and rubbing challenges without a stated return-to-reference or recovery period.</x:v>
+      </x:c>
+      <x:c r="J30" s="30" t="str">
+        <x:v>Post-exposure retention only; defined reference/recovery not reported: Post-exposure response followed temperature, water-immersion and rubbing challenges without a stated return-to-reference or recovery period. Evidence: Performance was measured after 40 °C, −35 °C and 24-h water immersion/rubbing exposures.</x:v>
+      </x:c>
+      <x:c r="K30" s="30" t="str">
+        <x:v>PDF pp. 2–12; Figs. 1–8; Supplementary Figs. S1–S15 cited</x:v>
+      </x:c>
+      <x:c r="L30" s="30"/>
+      <x:c r="M30" s="30"/>
+      <x:c r="N30" s="30"/>
+    </x:row>
+    <x:row r="31" ht="36" hidden="0" customHeight="1">
+      <x:c r="A31" s="30" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B31" s="30" t="str">
+        <x:v>S089</x:v>
+      </x:c>
+      <x:c r="C31" s="30" t="str">
+        <x:v>Xiang et al. (2020)</x:v>
+      </x:c>
+      <x:c r="D31" s="30" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E31" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only</x:v>
+      </x:c>
+      <x:c r="F31" s="30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G31" s="30" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H31" s="30" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="I31" s="30" t="str">
+        <x:v>No post-exposure retention endpoint was coded.</x:v>
+      </x:c>
+      <x:c r="J31" s="30" t="str">
+        <x:v>In-exposure cross-sensitivity only: Conductivity was measured and reported across a stated 20–80 °C exposure.</x:v>
+      </x:c>
+      <x:c r="K31" s="30" t="str">
+        <x:v>PDF pp. 10–35 of available accepted manuscript; Figs. 1–10; Tables 1–2; Supplementary Tables S1–S2 cited</x:v>
+      </x:c>
+      <x:c r="L31" s="30"/>
+      <x:c r="M31" s="30"/>
+      <x:c r="N31" s="30"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -41216,7 +42636,7 @@
         <x:v>Include</x:v>
       </x:c>
       <x:c r="H76" s="12" t="str">
-        <x:v>The retained FDM-printed soft-PLA substrate/mask defines the active channel and prevents electrode–electrolyte contact; the completed flexible OECT is characterized experimentally and the paper explicitly frames wearable biosensing use.</x:v>
+        <x:v>Borderline primary inclusion: the complete soft-PLA OECT substrate/mask defines the active channel in a flexible platform explicitly designed for wearable biosensing; no on-body experiment was reported. Excluded in the strict sensitivity analysis.</x:v>
       </x:c>
       <x:c r="I76" s="12" t="str">
         <x:v>PDF pp. 1–7; Figs. 1, 3–4; Tables 1–2</x:v>
@@ -41248,7 +42668,7 @@
         <x:v>Include</x:v>
       </x:c>
       <x:c r="H77" s="12" t="str">
-        <x:v>Thermoplastic-filament FDM directly prints the PVDF/MWCNT sensing strip, which is tested as a reversible VOC chemiresistor and proposed for wearable form factors.</x:v>
+        <x:v>Borderline primary inclusion: FDM prints the complete flexible chemiresistive sensing strip, reversible vapour response is measured, and the article explicitly specifies wearable form factors; no on-body experiment was reported. Excluded in the strict sensitivity analysis.</x:v>
       </x:c>
       <x:c r="I77" s="12" t="str">
         <x:v>PDF pp. 1–8; Figs. 2, 6–11; Table 1</x:v>
@@ -44064,7 +45484,7 @@
         <x:v>FDM creates the retained substrate and mask; the mask defines the active channel and isolates source/drain contacts from electrolyte</x:v>
       </x:c>
       <x:c r="G80" s="12" t="str">
-        <x:v>Flexible/wearable biosensing platform; no on-body test</x:v>
+        <x:v>Borderline primary inclusion: complete flexible OECT platform; no on-body test; excluded in strict sensitivity analysis</x:v>
       </x:c>
       <x:c r="H80" s="12" t="str">
         <x:v>Yes</x:v>
@@ -44134,7 +45554,7 @@
         <x:v>FDM directly prints the active conductive nanocomposite strip</x:v>
       </x:c>
       <x:c r="G82" s="12" t="str">
-        <x:v>Wearable-relevant flexible form factor; no on-body test</x:v>
+        <x:v>Borderline primary inclusion: complete flexible chemiresistive strip; no on-body test; excluded in strict sensitivity analysis</x:v>
       </x:c>
       <x:c r="H82" s="12" t="str">
         <x:v>Yes</x:v>

</xml_diff>